<commit_message>
latest code after merge with Madhukar
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataBelgiumMKv01.xlsx
+++ b/Data/Hires/TestDataBelgiumMKv01.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{1E2B50EA-DC35-4781-B862-7527F9DD23ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F1DD8706-EC53-4DF4-93A3-B96D7171294A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="217">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -229,12 +229,10 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>Test failed for 'Hollie Turner' Employee:{10697705}Error: [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m
-Expected: [32m"BE Monthly"[39m
-Received: [31m"Please select a Belgium Pay Group"[39m</t>
-  </si>
-  <si>
-    <t>Failed</t>
+    <t>10697784</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
   <si>
     <t>751 Retail Team 1 (Rykec Puvyjo (10528834) (Inherited))</t>
@@ -246,10 +244,10 @@
     <t>Mr</t>
   </si>
   <si>
-    <t>Hollie</t>
-  </si>
-  <si>
-    <t>Turner</t>
+    <t>Nyasia</t>
+  </si>
+  <si>
+    <t>Murray</t>
   </si>
   <si>
     <t>Landline</t>
@@ -385,6 +383,9 @@
 Call log:
   [2m- waiting for locator('[aria-label="Search Workday "]')[22m
 </t>
+  </si>
+  <si>
+    <t>Failed</t>
   </si>
   <si>
     <t>751 Store Management (Rykec Puvyjo (10528834))</t>
@@ -768,7 +769,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1589,7 +1590,7 @@
       </c>
       <c r="L2" s="19">
         <f t="shared" ref="L2" ca="1" si="0">TODAY()-31</f>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M2" s="14" t="s">
         <v>69</v>
@@ -1623,7 +1624,7 @@
       </c>
       <c r="W2" s="23">
         <f t="shared" ref="W2" ca="1" si="1">L2</f>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X2" s="18" t="s">
         <v>80</v>
@@ -1675,7 +1676,7 @@
       </c>
       <c r="AN2" s="29">
         <f t="array" aca="1" ref="AN2:AN16" ca="1">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
-        <v>94324563617</v>
+        <v>52464079638</v>
       </c>
       <c r="AO2" s="14" t="s">
         <v>93</v>
@@ -1771,22 +1772,22 @@
         <v>116</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>69</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I3" s="18">
         <v>25041111</v>
@@ -1799,7 +1800,7 @@
       </c>
       <c r="L3" s="19">
         <f t="shared" ref="L3:L16" ca="1" si="2">TODAY()-31</f>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M3" s="14" t="s">
         <v>69</v>
@@ -1833,19 +1834,19 @@
       </c>
       <c r="W3" s="23">
         <f t="shared" ref="W3:W16" ca="1" si="3">L3</f>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X3" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y3" s="24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="Z3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AA3" s="25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AB3" t="s">
         <v>84</v>
@@ -1860,20 +1861,20 @@
         <v>35</v>
       </c>
       <c r="AF3" s="14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AG3" t="s">
         <v>87</v>
       </c>
       <c r="AH3" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AI3" s="18" t="s">
         <v>89</v>
       </c>
       <c r="AJ3" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AK3" s="1">
         <v>251</v>
@@ -1886,23 +1887,23 @@
       </c>
       <c r="AN3" s="29">
         <f ca="1"/>
-        <v>93060018914</v>
+        <v>81569448446</v>
       </c>
       <c r="AO3" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP3" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AQ3" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR3" s="19">
         <f t="shared" ref="AR3:AR16" ca="1" si="4">AH3</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AS3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AT3" s="30">
         <v>35591</v>
@@ -1929,10 +1930,10 @@
         <v>69</v>
       </c>
       <c r="BB3" s="34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="BC3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="BD3" s="14" t="s">
         <v>102</v>
@@ -1953,10 +1954,10 @@
         <v>107</v>
       </c>
       <c r="BJ3" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK3" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL3" s="31" t="s">
         <v>110</v>
@@ -1976,7 +1977,7 @@
     </row>
     <row r="4" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="13" t="s">
@@ -1989,10 +1990,10 @@
         <v>70</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I4" s="18">
         <v>25041111</v>
@@ -2005,7 +2006,7 @@
       </c>
       <c r="L4" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M4" s="14" t="s">
         <v>69</v>
@@ -2039,7 +2040,7 @@
       </c>
       <c r="W4" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X4" s="18" t="s">
         <v>80</v>
@@ -2051,10 +2052,10 @@
         <v>82</v>
       </c>
       <c r="AA4" s="25" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AB4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC4" s="1" t="s">
         <v>85</v>
@@ -2081,7 +2082,7 @@
         <v>90</v>
       </c>
       <c r="AK4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AL4" s="28" t="s">
         <v>69</v>
@@ -2091,7 +2092,7 @@
       </c>
       <c r="AN4" s="29">
         <f ca="1"/>
-        <v>89688912606</v>
+        <v>19431753549</v>
       </c>
       <c r="AO4" s="14" t="s">
         <v>93</v>
@@ -2158,10 +2159,10 @@
         <v>107</v>
       </c>
       <c r="BJ4" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK4" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL4" s="31" t="s">
         <v>110</v>
@@ -2176,28 +2177,28 @@
         <v>113</v>
       </c>
       <c r="BP4" s="33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>69</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I5" s="18">
         <v>25041111</v>
@@ -2210,7 +2211,7 @@
       </c>
       <c r="L5" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M5" s="14" t="s">
         <v>69</v>
@@ -2244,19 +2245,19 @@
       </c>
       <c r="W5" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X5" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y5" s="24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Z5" t="s">
         <v>82</v>
       </c>
       <c r="AA5" s="25" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="AB5" t="s">
         <v>84</v>
@@ -2271,7 +2272,7 @@
         <v>35</v>
       </c>
       <c r="AF5" s="14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AG5" t="s">
         <v>87</v>
@@ -2283,7 +2284,7 @@
         <v>89</v>
       </c>
       <c r="AJ5" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AK5" s="1">
         <v>251</v>
@@ -2296,7 +2297,7 @@
       </c>
       <c r="AN5" s="29">
         <f ca="1"/>
-        <v>21298998942</v>
+        <v>91305818781</v>
       </c>
       <c r="AO5" s="14" t="s">
         <v>93</v>
@@ -2312,7 +2313,7 @@
         <v>N/A</v>
       </c>
       <c r="AS5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AT5" s="30">
         <v>35591</v>
@@ -2339,10 +2340,10 @@
         <v>69</v>
       </c>
       <c r="BB5" s="34" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="BC5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="BD5" s="14" t="s">
         <v>102</v>
@@ -2363,10 +2364,10 @@
         <v>107</v>
       </c>
       <c r="BJ5" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK5" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL5" s="31" t="s">
         <v>110</v>
@@ -2386,7 +2387,7 @@
     </row>
     <row r="6" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="13" t="s">
@@ -2399,10 +2400,10 @@
         <v>70</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I6" s="18">
         <v>25041111</v>
@@ -2415,7 +2416,7 @@
       </c>
       <c r="L6" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M6" s="14" t="s">
         <v>69</v>
@@ -2449,7 +2450,7 @@
       </c>
       <c r="W6" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X6" s="18" t="s">
         <v>80</v>
@@ -2458,13 +2459,13 @@
         <v>81</v>
       </c>
       <c r="Z6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AA6" s="25" t="s">
         <v>83</v>
       </c>
       <c r="AB6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC6" s="1" t="s">
         <v>85</v>
@@ -2483,7 +2484,7 @@
       </c>
       <c r="AH6" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AI6" s="18" t="s">
         <v>89</v>
@@ -2492,7 +2493,7 @@
         <v>90</v>
       </c>
       <c r="AK6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AL6" s="28" t="s">
         <v>69</v>
@@ -2502,20 +2503,20 @@
       </c>
       <c r="AN6" s="29">
         <f ca="1"/>
-        <v>34812002012</v>
+        <v>28307817987</v>
       </c>
       <c r="AO6" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP6" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AQ6" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR6" s="19">
         <f t="shared" ca="1" si="4"/>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AS6" t="s">
         <v>96</v>
@@ -2569,10 +2570,10 @@
         <v>107</v>
       </c>
       <c r="BJ6" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK6" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL6" s="31" t="s">
         <v>110</v>
@@ -2587,16 +2588,16 @@
         <v>113</v>
       </c>
       <c r="BP6" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>69</v>
@@ -2605,10 +2606,10 @@
         <v>70</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I7" s="18">
         <v>25041111</v>
@@ -2621,7 +2622,7 @@
       </c>
       <c r="L7" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M7" s="14" t="s">
         <v>69</v>
@@ -2655,22 +2656,22 @@
       </c>
       <c r="W7" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X7" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y7" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="Z7" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="AB7" s="37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC7" s="1" t="s">
         <v>85</v>
@@ -2694,7 +2695,7 @@
         <v>89</v>
       </c>
       <c r="AJ7" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AK7" s="1">
         <v>251</v>
@@ -2707,7 +2708,7 @@
       </c>
       <c r="AN7" s="29">
         <f ca="1"/>
-        <v>41725020278</v>
+        <v>90116436576</v>
       </c>
       <c r="AO7" s="14" t="s">
         <v>93</v>
@@ -2750,10 +2751,10 @@
         <v>69</v>
       </c>
       <c r="BB7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BC7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BD7" s="14" t="s">
         <v>102</v>
@@ -2774,10 +2775,10 @@
         <v>107</v>
       </c>
       <c r="BJ7" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK7" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL7" s="31" t="s">
         <v>110</v>
@@ -2792,16 +2793,16 @@
         <v>113</v>
       </c>
       <c r="BP7" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>69</v>
@@ -2810,10 +2811,10 @@
         <v>70</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
@@ -2826,7 +2827,7 @@
       </c>
       <c r="L8" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M8" s="14" t="s">
         <v>69</v>
@@ -2860,19 +2861,19 @@
       </c>
       <c r="W8" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X8" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="Z8" s="36" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AB8" s="37" t="s">
         <v>84</v>
@@ -2894,13 +2895,13 @@
       </c>
       <c r="AH8" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AI8" s="18" t="s">
         <v>89</v>
       </c>
       <c r="AJ8" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AK8" s="1">
         <v>251</v>
@@ -2913,20 +2914,20 @@
       </c>
       <c r="AN8" s="29">
         <f ca="1"/>
-        <v>29419178734</v>
+        <v>88397911747</v>
       </c>
       <c r="AO8" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP8" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AQ8" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR8" s="19">
         <f t="shared" ca="1" si="4"/>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AS8" t="s">
         <v>96</v>
@@ -2956,10 +2957,10 @@
         <v>69</v>
       </c>
       <c r="BB8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="BC8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="BD8" s="14" t="s">
         <v>102</v>
@@ -2980,10 +2981,10 @@
         <v>107</v>
       </c>
       <c r="BJ8" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK8" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL8" s="31" t="s">
         <v>110</v>
@@ -3003,11 +3004,11 @@
     </row>
     <row r="9" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>69</v>
@@ -3016,10 +3017,10 @@
         <v>70</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
@@ -3032,7 +3033,7 @@
       </c>
       <c r="L9" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M9" s="14" t="s">
         <v>69</v>
@@ -3066,22 +3067,22 @@
       </c>
       <c r="W9" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X9" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y9" s="24" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Z9" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AB9" s="37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC9" s="1" t="s">
         <v>85</v>
@@ -3105,7 +3106,7 @@
         <v>89</v>
       </c>
       <c r="AJ9" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AK9" s="1">
         <v>251</v>
@@ -3118,7 +3119,7 @@
       </c>
       <c r="AN9" s="29">
         <f ca="1"/>
-        <v>57853992991</v>
+        <v>57149063321</v>
       </c>
       <c r="AO9" s="14" t="s">
         <v>93</v>
@@ -3161,10 +3162,10 @@
         <v>69</v>
       </c>
       <c r="BB9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="BC9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="BD9" s="14" t="s">
         <v>102</v>
@@ -3185,10 +3186,10 @@
         <v>107</v>
       </c>
       <c r="BJ9" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK9" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL9" s="31" t="s">
         <v>110</v>
@@ -3203,12 +3204,12 @@
         <v>113</v>
       </c>
       <c r="BP9" s="33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13" t="s">
@@ -3221,10 +3222,10 @@
         <v>70</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
@@ -3237,7 +3238,7 @@
       </c>
       <c r="L10" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M10" s="14" t="s">
         <v>69</v>
@@ -3271,7 +3272,7 @@
       </c>
       <c r="W10" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X10" s="18" t="s">
         <v>80</v>
@@ -3280,19 +3281,19 @@
         <v>81</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AB10" s="37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC10" s="1" t="s">
         <v>85</v>
       </c>
       <c r="AD10" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
@@ -3305,7 +3306,7 @@
       </c>
       <c r="AH10" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AI10" s="18" t="s">
         <v>89</v>
@@ -3314,7 +3315,7 @@
         <v>90</v>
       </c>
       <c r="AK10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AL10" s="28" t="s">
         <v>69</v>
@@ -3324,20 +3325,20 @@
       </c>
       <c r="AN10" s="29">
         <f ca="1"/>
-        <v>39119527441</v>
+        <v>74848109800</v>
       </c>
       <c r="AO10" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP10" s="20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AQ10" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR10" s="19">
         <f t="shared" ca="1" si="4"/>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AS10" t="s">
         <v>96</v>
@@ -3391,10 +3392,10 @@
         <v>107</v>
       </c>
       <c r="BJ10" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK10" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL10" s="31" t="s">
         <v>110</v>
@@ -3409,12 +3410,12 @@
         <v>113</v>
       </c>
       <c r="BP10" s="38" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13" t="s">
@@ -3427,10 +3428,10 @@
         <v>70</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
@@ -3443,7 +3444,7 @@
       </c>
       <c r="L11" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M11" s="14" t="s">
         <v>69</v>
@@ -3477,7 +3478,7 @@
       </c>
       <c r="W11" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X11" s="18" t="s">
         <v>80</v>
@@ -3489,7 +3490,7 @@
         <v>82</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AB11" s="38" t="s">
         <v>84</v>
@@ -3519,7 +3520,7 @@
         <v>90</v>
       </c>
       <c r="AK11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AL11" s="28" t="s">
         <v>69</v>
@@ -3529,7 +3530,7 @@
       </c>
       <c r="AN11" s="29">
         <f ca="1"/>
-        <v>49343930312</v>
+        <v>83735190113</v>
       </c>
       <c r="AO11" s="14" t="s">
         <v>93</v>
@@ -3572,10 +3573,10 @@
         <v>69</v>
       </c>
       <c r="BB11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="BC11" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="BD11" s="14" t="s">
         <v>102</v>
@@ -3596,10 +3597,10 @@
         <v>107</v>
       </c>
       <c r="BJ11" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK11" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL11" s="31" t="s">
         <v>110</v>
@@ -3619,7 +3620,7 @@
     </row>
     <row r="12" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13" t="s">
@@ -3632,10 +3633,10 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
@@ -3648,7 +3649,7 @@
       </c>
       <c r="L12" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M12" s="14" t="s">
         <v>69</v>
@@ -3682,7 +3683,7 @@
       </c>
       <c r="W12" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X12" s="18" t="s">
         <v>80</v>
@@ -3694,10 +3695,10 @@
         <v>82</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AB12" s="37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC12" s="1" t="s">
         <v>85</v>
@@ -3724,7 +3725,7 @@
         <v>90</v>
       </c>
       <c r="AK12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AL12" s="28" t="s">
         <v>69</v>
@@ -3734,7 +3735,7 @@
       </c>
       <c r="AN12" s="29">
         <f ca="1"/>
-        <v>55342346241</v>
+        <v>91076330092</v>
       </c>
       <c r="AO12" s="14" t="s">
         <v>93</v>
@@ -3801,10 +3802,10 @@
         <v>107</v>
       </c>
       <c r="BJ12" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK12" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL12" s="31" t="s">
         <v>110</v>
@@ -3819,12 +3820,12 @@
         <v>113</v>
       </c>
       <c r="BP12" s="38" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="13" t="s">
@@ -3837,10 +3838,10 @@
         <v>70</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
@@ -3853,7 +3854,7 @@
       </c>
       <c r="L13" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M13" s="14" t="s">
         <v>69</v>
@@ -3887,7 +3888,7 @@
       </c>
       <c r="W13" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X13" s="18" t="s">
         <v>80</v>
@@ -3896,10 +3897,10 @@
         <v>81</v>
       </c>
       <c r="Z13" s="36" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AB13" s="37" t="s">
         <v>84</v>
@@ -3921,7 +3922,7 @@
       </c>
       <c r="AH13" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AI13" s="18" t="s">
         <v>89</v>
@@ -3930,7 +3931,7 @@
         <v>90</v>
       </c>
       <c r="AK13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AL13" s="28" t="s">
         <v>69</v>
@@ -3940,20 +3941,20 @@
       </c>
       <c r="AN13" s="29">
         <f ca="1"/>
-        <v>14287234855</v>
+        <v>12772211778</v>
       </c>
       <c r="AO13" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP13" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AQ13" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR13" s="19">
         <f t="shared" ca="1" si="4"/>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AS13" t="s">
         <v>96</v>
@@ -3983,10 +3984,10 @@
         <v>69</v>
       </c>
       <c r="BB13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="BD13" s="14" t="s">
         <v>102</v>
@@ -4007,10 +4008,10 @@
         <v>107</v>
       </c>
       <c r="BJ13" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK13" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL13" s="31" t="s">
         <v>110</v>
@@ -4030,7 +4031,7 @@
     </row>
     <row r="14" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="13" t="s">
@@ -4043,10 +4044,10 @@
         <v>70</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
@@ -4059,7 +4060,7 @@
       </c>
       <c r="L14" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M14" s="14" t="s">
         <v>69</v>
@@ -4093,7 +4094,7 @@
       </c>
       <c r="W14" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X14" s="18" t="s">
         <v>80</v>
@@ -4105,10 +4106,10 @@
         <v>82</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AB14" s="37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC14" s="1" t="s">
         <v>85</v>
@@ -4135,7 +4136,7 @@
         <v>90</v>
       </c>
       <c r="AK14" s="38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AL14" s="28" t="s">
         <v>69</v>
@@ -4145,7 +4146,7 @@
       </c>
       <c r="AN14" s="29">
         <f ca="1"/>
-        <v>71085990665</v>
+        <v>61588847689</v>
       </c>
       <c r="AO14" s="14" t="s">
         <v>93</v>
@@ -4212,10 +4213,10 @@
         <v>107</v>
       </c>
       <c r="BJ14" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK14" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL14" s="31" t="s">
         <v>110</v>
@@ -4230,12 +4231,12 @@
         <v>113</v>
       </c>
       <c r="BP14" s="38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13" t="s">
@@ -4248,10 +4249,10 @@
         <v>70</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
@@ -4264,7 +4265,7 @@
       </c>
       <c r="L15" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M15" s="14" t="s">
         <v>69</v>
@@ -4298,7 +4299,7 @@
       </c>
       <c r="W15" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X15" s="18" t="s">
         <v>80</v>
@@ -4307,13 +4308,13 @@
         <v>81</v>
       </c>
       <c r="Z15" s="36" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AA15" s="25" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="AB15" s="37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC15" s="1" t="s">
         <v>85</v>
@@ -4332,7 +4333,7 @@
       </c>
       <c r="AH15" s="19">
         <f ca="1">TODAY()+365</f>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AI15" s="18" t="s">
         <v>89</v>
@@ -4341,7 +4342,7 @@
         <v>90</v>
       </c>
       <c r="AK15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AL15" s="28" t="s">
         <v>69</v>
@@ -4351,20 +4352,20 @@
       </c>
       <c r="AN15" s="29">
         <f ca="1"/>
-        <v>87855427514</v>
+        <v>62719197684</v>
       </c>
       <c r="AO15" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP15" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AQ15" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR15" s="19">
         <f t="shared" ca="1" si="4"/>
-        <v>46085</v>
+        <v>46087</v>
       </c>
       <c r="AS15" t="s">
         <v>96</v>
@@ -4394,10 +4395,10 @@
         <v>69</v>
       </c>
       <c r="BB15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="BC15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="BD15" s="14" t="s">
         <v>102</v>
@@ -4418,10 +4419,10 @@
         <v>107</v>
       </c>
       <c r="BJ15" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK15" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL15" s="31" t="s">
         <v>110</v>
@@ -4436,16 +4437,16 @@
         <v>113</v>
       </c>
       <c r="BP15" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>69</v>
@@ -4454,10 +4455,10 @@
         <v>70</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
@@ -4470,7 +4471,7 @@
       </c>
       <c r="L16" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="M16" s="14" t="s">
         <v>69</v>
@@ -4504,19 +4505,19 @@
       </c>
       <c r="W16" s="23">
         <f t="shared" ca="1" si="3"/>
-        <v>45689</v>
+        <v>45691</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z16" s="38" t="s">
         <v>82</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AB16" s="37" t="s">
         <v>84</v>
@@ -4543,7 +4544,7 @@
         <v>89</v>
       </c>
       <c r="AJ16" s="18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AK16" s="1">
         <v>251</v>
@@ -4556,7 +4557,7 @@
       </c>
       <c r="AN16" s="29">
         <f ca="1"/>
-        <v>42677516640</v>
+        <v>28598841032</v>
       </c>
       <c r="AO16" s="14" t="s">
         <v>93</v>
@@ -4623,10 +4624,10 @@
         <v>107</v>
       </c>
       <c r="BJ16" s="31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BK16" s="31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BL16" s="31" t="s">
         <v>110</v>

</xml_diff>

<commit_message>
latest code for slovenia 60% completd.
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataBelgiumMKv01.xlsx
+++ b/Data/Hires/TestDataBelgiumMKv01.xlsx
@@ -1,35 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F1DD8706-EC53-4DF4-93A3-B96D7171294A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="216">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -229,10 +214,250 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10697784</t>
-  </si>
-  <si>
-    <t>Passed</t>
+    <t xml:space="preserve">Test failed for 'Carter Smith' Employee:{undefined}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByLabel('My Tasks Items').first()[22m
+[2m  -   locator resolved to &lt;button class="wdappchrome-w" data-automation-id="inbox_…&gt;…&lt;/button&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #1[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #2[22m
+[2m  -   waiting 20ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #3[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #4[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #5[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #6[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #7[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #8[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #9[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #10[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #11[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #12[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #13[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #14[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #15[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #16[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #17[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #18[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #19[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #20[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #21[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #22[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #23[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #24[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #25[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #26[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #27[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #28[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #29[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #30[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #31[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #32[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #33[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #34[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #35[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #36[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #37[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #38[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #39[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #40[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #41[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #42[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #43[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #44[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #45[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #46[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #47[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #48[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #49[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #50[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #51[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #52[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #53[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #54[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #55[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #56[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #57[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #58[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is not visible[22m
+[2m  - retrying click action, attempt #59[22m
+[2m  -   waiting 500ms[22m
+</t>
+  </si>
+  <si>
+    <t>Failed</t>
   </si>
   <si>
     <t>751 Retail Team 1 (Rykec Puvyjo (10528834) (Inherited))</t>
@@ -244,10 +469,10 @@
     <t>Mr</t>
   </si>
   <si>
-    <t>Nyasia</t>
-  </si>
-  <si>
-    <t>Murray</t>
+    <t>Carter</t>
+  </si>
+  <si>
+    <t>Farrell</t>
   </si>
   <si>
     <t>Landline</t>
@@ -385,9 +610,6 @@
 </t>
   </si>
   <si>
-    <t>Failed</t>
-  </si>
-  <si>
     <t>751 Store Management (Rykec Puvyjo (10528834))</t>
   </si>
   <si>
@@ -688,58 +910,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color indexed="8"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color indexed="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FF4A4A4A"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FF1F1F1F"/>
+      <family val="3"/>
       <sz val="6"/>
-      <color rgb="FF1F1F1F"/>
       <name val="Courier New"/>
-      <family val="3"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FF800000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
@@ -751,25 +973,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -788,12 +1010,8 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -803,25 +1021,15 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -832,22 +1040,14 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left style="thin"/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -862,29 +1062,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <left style="thin"/>
+      <right style="thin"/>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1276,9 +1464,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BP16"/>
-  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1348,7 +1536,7 @@
     <col min="68" max="68" width="16.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.5" customHeight="1" spans="1:68" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1554,7 +1742,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>65</v>
       </c>
@@ -1589,7 +1777,7 @@
         <v>74</v>
       </c>
       <c r="L2" s="19">
-        <f t="shared" ref="L2" ca="1" si="0">TODAY()-31</f>
+        <f t="shared" ref="L2" si="0">TODAY()-31</f>
         <v>45691</v>
       </c>
       <c r="M2" s="14" t="s">
@@ -1623,7 +1811,7 @@
         <v>74</v>
       </c>
       <c r="W2" s="23">
-        <f t="shared" ref="W2" ca="1" si="1">L2</f>
+        <f t="shared" ref="W2" si="1">L2</f>
         <v>45691</v>
       </c>
       <c r="X2" s="18" t="s">
@@ -1675,7 +1863,7 @@
         <v>92</v>
       </c>
       <c r="AN2" s="29">
-        <f t="array" aca="1" ref="AN2:AN16" ca="1">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
+        <f t="array" ref="AN2:AN16">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
         <v>52464079638</v>
       </c>
       <c r="AO2" s="14" t="s">
@@ -1687,9 +1875,9 @@
       <c r="AQ2" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR2" s="19" t="str">
+      <c r="AR2" s="19">
         <f>AH2</f>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS2" t="s">
         <v>96</v>
@@ -1764,7 +1952,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>115</v>
       </c>
@@ -1772,22 +1960,22 @@
         <v>116</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="E3" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="H3" s="17" t="s">
         <v>120</v>
-      </c>
-      <c r="H3" s="17" t="s">
-        <v>121</v>
       </c>
       <c r="I3" s="18">
         <v>25041111</v>
@@ -1799,7 +1987,7 @@
         <v>74</v>
       </c>
       <c r="L3" s="19">
-        <f t="shared" ref="L3:L16" ca="1" si="2">TODAY()-31</f>
+        <f t="shared" ref="L3:L16" si="2">TODAY()-31</f>
         <v>45691</v>
       </c>
       <c r="M3" s="14" t="s">
@@ -1833,20 +2021,20 @@
         <v>74</v>
       </c>
       <c r="W3" s="23">
-        <f t="shared" ref="W3:W16" ca="1" si="3">L3</f>
+        <f t="shared" ref="W3:W16" si="3">L3</f>
         <v>45691</v>
       </c>
       <c r="X3" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y3" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="Z3" t="s">
         <v>122</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" s="25" t="s">
         <v>123</v>
-      </c>
-      <c r="AA3" s="25" t="s">
-        <v>124</v>
       </c>
       <c r="AB3" t="s">
         <v>84</v>
@@ -1861,20 +2049,20 @@
         <v>35</v>
       </c>
       <c r="AF3" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG3" t="s">
         <v>87</v>
       </c>
       <c r="AH3" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46087</v>
       </c>
       <c r="AI3" s="18" t="s">
         <v>89</v>
       </c>
       <c r="AJ3" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK3" s="1">
         <v>251</v>
@@ -1886,24 +2074,23 @@
         <v>92</v>
       </c>
       <c r="AN3" s="29">
-        <f ca="1"/>
         <v>81569448446</v>
       </c>
       <c r="AO3" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP3" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AQ3" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR3" s="19">
-        <f t="shared" ref="AR3:AR16" ca="1" si="4">AH3</f>
+        <f t="shared" ref="AR3:AR16" si="4">AH3</f>
         <v>46087</v>
       </c>
       <c r="AS3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AT3" s="30">
         <v>35591</v>
@@ -1930,10 +2117,10 @@
         <v>69</v>
       </c>
       <c r="BB3" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="BC3" t="s">
         <v>128</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>129</v>
       </c>
       <c r="BD3" s="14" t="s">
         <v>102</v>
@@ -1954,10 +2141,10 @@
         <v>107</v>
       </c>
       <c r="BJ3" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK3" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK3" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL3" s="31" t="s">
         <v>110</v>
@@ -1975,9 +2162,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="13" t="s">
@@ -1990,10 +2177,10 @@
         <v>70</v>
       </c>
       <c r="G4" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="17" t="s">
         <v>133</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>134</v>
       </c>
       <c r="I4" s="18">
         <v>25041111</v>
@@ -2005,7 +2192,7 @@
         <v>74</v>
       </c>
       <c r="L4" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M4" s="14" t="s">
@@ -2039,7 +2226,7 @@
         <v>74</v>
       </c>
       <c r="W4" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X4" s="18" t="s">
@@ -2052,10 +2239,10 @@
         <v>82</v>
       </c>
       <c r="AA4" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="AB4" t="s">
         <v>135</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>136</v>
       </c>
       <c r="AC4" s="1" t="s">
         <v>85</v>
@@ -2082,7 +2269,7 @@
         <v>90</v>
       </c>
       <c r="AK4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AL4" s="28" t="s">
         <v>69</v>
@@ -2091,7 +2278,6 @@
         <v>92</v>
       </c>
       <c r="AN4" s="29">
-        <f ca="1"/>
         <v>19431753549</v>
       </c>
       <c r="AO4" s="14" t="s">
@@ -2103,9 +2289,9 @@
       <c r="AQ4" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR4" s="19" t="str">
+      <c r="AR4" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS4" t="s">
         <v>96</v>
@@ -2159,10 +2345,10 @@
         <v>107</v>
       </c>
       <c r="BJ4" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK4" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK4" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL4" s="31" t="s">
         <v>110</v>
@@ -2177,28 +2363,28 @@
         <v>113</v>
       </c>
       <c r="BP4" s="33" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="5" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>119</v>
-      </c>
       <c r="G5" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="H5" s="17" t="s">
         <v>140</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>141</v>
       </c>
       <c r="I5" s="18">
         <v>25041111</v>
@@ -2210,7 +2396,7 @@
         <v>74</v>
       </c>
       <c r="L5" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M5" s="14" t="s">
@@ -2244,20 +2430,20 @@
         <v>74</v>
       </c>
       <c r="W5" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X5" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y5" s="24" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Z5" t="s">
         <v>82</v>
       </c>
       <c r="AA5" s="25" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AB5" t="s">
         <v>84</v>
@@ -2272,7 +2458,7 @@
         <v>35</v>
       </c>
       <c r="AF5" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AG5" t="s">
         <v>87</v>
@@ -2284,7 +2470,7 @@
         <v>89</v>
       </c>
       <c r="AJ5" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK5" s="1">
         <v>251</v>
@@ -2296,7 +2482,6 @@
         <v>92</v>
       </c>
       <c r="AN5" s="29">
-        <f ca="1"/>
         <v>91305818781</v>
       </c>
       <c r="AO5" s="14" t="s">
@@ -2308,12 +2493,12 @@
       <c r="AQ5" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR5" s="19" t="str">
+      <c r="AR5" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AT5" s="30">
         <v>35591</v>
@@ -2340,10 +2525,10 @@
         <v>69</v>
       </c>
       <c r="BB5" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="BC5" t="s">
         <v>144</v>
-      </c>
-      <c r="BC5" t="s">
-        <v>145</v>
       </c>
       <c r="BD5" s="14" t="s">
         <v>102</v>
@@ -2364,10 +2549,10 @@
         <v>107</v>
       </c>
       <c r="BJ5" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK5" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK5" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL5" s="31" t="s">
         <v>110</v>
@@ -2385,9 +2570,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="13" t="s">
@@ -2400,10 +2585,10 @@
         <v>70</v>
       </c>
       <c r="G6" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6" s="17" t="s">
         <v>147</v>
-      </c>
-      <c r="H6" s="17" t="s">
-        <v>148</v>
       </c>
       <c r="I6" s="18">
         <v>25041111</v>
@@ -2415,7 +2600,7 @@
         <v>74</v>
       </c>
       <c r="L6" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M6" s="14" t="s">
@@ -2449,7 +2634,7 @@
         <v>74</v>
       </c>
       <c r="W6" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X6" s="18" t="s">
@@ -2459,13 +2644,13 @@
         <v>81</v>
       </c>
       <c r="Z6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AA6" s="25" t="s">
         <v>83</v>
       </c>
       <c r="AB6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC6" s="1" t="s">
         <v>85</v>
@@ -2483,7 +2668,7 @@
         <v>87</v>
       </c>
       <c r="AH6" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46087</v>
       </c>
       <c r="AI6" s="18" t="s">
@@ -2493,7 +2678,7 @@
         <v>90</v>
       </c>
       <c r="AK6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AL6" s="28" t="s">
         <v>69</v>
@@ -2502,20 +2687,19 @@
         <v>92</v>
       </c>
       <c r="AN6" s="29">
-        <f ca="1"/>
         <v>28307817987</v>
       </c>
       <c r="AO6" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP6" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AQ6" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR6" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46087</v>
       </c>
       <c r="AS6" t="s">
@@ -2570,10 +2754,10 @@
         <v>107</v>
       </c>
       <c r="BJ6" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK6" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK6" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL6" s="31" t="s">
         <v>110</v>
@@ -2588,16 +2772,16 @@
         <v>113</v>
       </c>
       <c r="BP6" s="33" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="7" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>69</v>
@@ -2606,10 +2790,10 @@
         <v>70</v>
       </c>
       <c r="G7" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="H7" s="17" t="s">
         <v>153</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>154</v>
       </c>
       <c r="I7" s="18">
         <v>25041111</v>
@@ -2621,7 +2805,7 @@
         <v>74</v>
       </c>
       <c r="L7" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M7" s="14" t="s">
@@ -2655,23 +2839,23 @@
         <v>74</v>
       </c>
       <c r="W7" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X7" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y7" s="24" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Z7" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AB7" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC7" s="1" t="s">
         <v>85</v>
@@ -2695,7 +2879,7 @@
         <v>89</v>
       </c>
       <c r="AJ7" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK7" s="1">
         <v>251</v>
@@ -2707,7 +2891,6 @@
         <v>92</v>
       </c>
       <c r="AN7" s="29">
-        <f ca="1"/>
         <v>90116436576</v>
       </c>
       <c r="AO7" s="14" t="s">
@@ -2719,9 +2902,9 @@
       <c r="AQ7" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR7" s="19" t="str">
+      <c r="AR7" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS7" t="s">
         <v>96</v>
@@ -2751,10 +2934,10 @@
         <v>69</v>
       </c>
       <c r="BB7" t="s">
+        <v>156</v>
+      </c>
+      <c r="BC7" t="s">
         <v>157</v>
-      </c>
-      <c r="BC7" t="s">
-        <v>158</v>
       </c>
       <c r="BD7" s="14" t="s">
         <v>102</v>
@@ -2775,10 +2958,10 @@
         <v>107</v>
       </c>
       <c r="BJ7" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK7" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK7" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL7" s="31" t="s">
         <v>110</v>
@@ -2793,16 +2976,16 @@
         <v>113</v>
       </c>
       <c r="BP7" s="33" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
-    <row r="8" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>69</v>
@@ -2811,10 +2994,10 @@
         <v>70</v>
       </c>
       <c r="G8" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="H8" s="17" t="s">
         <v>160</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>161</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
@@ -2826,7 +3009,7 @@
         <v>74</v>
       </c>
       <c r="L8" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M8" s="14" t="s">
@@ -2860,20 +3043,20 @@
         <v>74</v>
       </c>
       <c r="W8" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X8" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y8" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="Z8" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="AA8" s="25" t="s">
         <v>162</v>
-      </c>
-      <c r="Z8" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="AA8" s="25" t="s">
-        <v>163</v>
       </c>
       <c r="AB8" s="37" t="s">
         <v>84</v>
@@ -2894,14 +3077,14 @@
         <v>87</v>
       </c>
       <c r="AH8" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46087</v>
       </c>
       <c r="AI8" s="18" t="s">
         <v>89</v>
       </c>
       <c r="AJ8" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK8" s="1">
         <v>251</v>
@@ -2913,20 +3096,19 @@
         <v>92</v>
       </c>
       <c r="AN8" s="29">
-        <f ca="1"/>
         <v>88397911747</v>
       </c>
       <c r="AO8" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP8" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AQ8" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR8" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46087</v>
       </c>
       <c r="AS8" t="s">
@@ -2957,10 +3139,10 @@
         <v>69</v>
       </c>
       <c r="BB8" t="s">
+        <v>163</v>
+      </c>
+      <c r="BC8" t="s">
         <v>164</v>
-      </c>
-      <c r="BC8" t="s">
-        <v>165</v>
       </c>
       <c r="BD8" s="14" t="s">
         <v>102</v>
@@ -2981,10 +3163,10 @@
         <v>107</v>
       </c>
       <c r="BJ8" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK8" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK8" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL8" s="31" t="s">
         <v>110</v>
@@ -3002,13 +3184,13 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>69</v>
@@ -3017,10 +3199,10 @@
         <v>70</v>
       </c>
       <c r="G9" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="H9" s="17" t="s">
         <v>167</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>168</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
@@ -3032,7 +3214,7 @@
         <v>74</v>
       </c>
       <c r="L9" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M9" s="14" t="s">
@@ -3066,23 +3248,23 @@
         <v>74</v>
       </c>
       <c r="W9" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X9" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y9" s="24" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Z9" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AB9" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC9" s="1" t="s">
         <v>85</v>
@@ -3106,7 +3288,7 @@
         <v>89</v>
       </c>
       <c r="AJ9" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK9" s="1">
         <v>251</v>
@@ -3118,7 +3300,6 @@
         <v>92</v>
       </c>
       <c r="AN9" s="29">
-        <f ca="1"/>
         <v>57149063321</v>
       </c>
       <c r="AO9" s="14" t="s">
@@ -3130,9 +3311,9 @@
       <c r="AQ9" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR9" s="19" t="str">
+      <c r="AR9" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS9" t="s">
         <v>96</v>
@@ -3162,10 +3343,10 @@
         <v>69</v>
       </c>
       <c r="BB9" t="s">
+        <v>170</v>
+      </c>
+      <c r="BC9" t="s">
         <v>171</v>
-      </c>
-      <c r="BC9" t="s">
-        <v>172</v>
       </c>
       <c r="BD9" s="14" t="s">
         <v>102</v>
@@ -3186,10 +3367,10 @@
         <v>107</v>
       </c>
       <c r="BJ9" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK9" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK9" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL9" s="31" t="s">
         <v>110</v>
@@ -3204,12 +3385,12 @@
         <v>113</v>
       </c>
       <c r="BP9" s="33" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13" t="s">
@@ -3222,10 +3403,10 @@
         <v>70</v>
       </c>
       <c r="G10" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="H10" s="17" t="s">
         <v>174</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>175</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
@@ -3237,7 +3418,7 @@
         <v>74</v>
       </c>
       <c r="L10" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M10" s="14" t="s">
@@ -3271,7 +3452,7 @@
         <v>74</v>
       </c>
       <c r="W10" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X10" s="18" t="s">
@@ -3281,19 +3462,19 @@
         <v>81</v>
       </c>
       <c r="Z10" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA10" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="AA10" s="25" t="s">
-        <v>177</v>
-      </c>
       <c r="AB10" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC10" s="1" t="s">
         <v>85</v>
       </c>
       <c r="AD10" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
@@ -3305,7 +3486,7 @@
         <v>87</v>
       </c>
       <c r="AH10" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46087</v>
       </c>
       <c r="AI10" s="18" t="s">
@@ -3315,7 +3496,7 @@
         <v>90</v>
       </c>
       <c r="AK10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AL10" s="28" t="s">
         <v>69</v>
@@ -3324,20 +3505,19 @@
         <v>92</v>
       </c>
       <c r="AN10" s="29">
-        <f ca="1"/>
         <v>74848109800</v>
       </c>
       <c r="AO10" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP10" s="20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AQ10" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR10" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46087</v>
       </c>
       <c r="AS10" t="s">
@@ -3392,10 +3572,10 @@
         <v>107</v>
       </c>
       <c r="BJ10" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK10" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK10" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL10" s="31" t="s">
         <v>110</v>
@@ -3410,12 +3590,12 @@
         <v>113</v>
       </c>
       <c r="BP10" s="38" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="11" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>180</v>
-      </c>
-    </row>
-    <row r="11" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>181</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13" t="s">
@@ -3428,10 +3608,10 @@
         <v>70</v>
       </c>
       <c r="G11" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="17" t="s">
         <v>182</v>
-      </c>
-      <c r="H11" s="17" t="s">
-        <v>183</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
@@ -3443,7 +3623,7 @@
         <v>74</v>
       </c>
       <c r="L11" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M11" s="14" t="s">
@@ -3477,7 +3657,7 @@
         <v>74</v>
       </c>
       <c r="W11" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X11" s="18" t="s">
@@ -3490,7 +3670,7 @@
         <v>82</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AB11" s="38" t="s">
         <v>84</v>
@@ -3520,7 +3700,7 @@
         <v>90</v>
       </c>
       <c r="AK11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AL11" s="28" t="s">
         <v>69</v>
@@ -3529,7 +3709,6 @@
         <v>92</v>
       </c>
       <c r="AN11" s="29">
-        <f ca="1"/>
         <v>83735190113</v>
       </c>
       <c r="AO11" s="14" t="s">
@@ -3541,9 +3720,9 @@
       <c r="AQ11" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR11" s="19" t="str">
+      <c r="AR11" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS11" t="s">
         <v>96</v>
@@ -3573,10 +3752,10 @@
         <v>69</v>
       </c>
       <c r="BB11" t="s">
+        <v>185</v>
+      </c>
+      <c r="BC11" t="s">
         <v>186</v>
-      </c>
-      <c r="BC11" t="s">
-        <v>187</v>
       </c>
       <c r="BD11" s="14" t="s">
         <v>102</v>
@@ -3597,10 +3776,10 @@
         <v>107</v>
       </c>
       <c r="BJ11" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK11" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK11" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL11" s="31" t="s">
         <v>110</v>
@@ -3618,9 +3797,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13" t="s">
@@ -3633,10 +3812,10 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="H12" s="17" t="s">
         <v>189</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>190</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
@@ -3648,7 +3827,7 @@
         <v>74</v>
       </c>
       <c r="L12" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M12" s="14" t="s">
@@ -3682,7 +3861,7 @@
         <v>74</v>
       </c>
       <c r="W12" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X12" s="18" t="s">
@@ -3695,10 +3874,10 @@
         <v>82</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AB12" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC12" s="1" t="s">
         <v>85</v>
@@ -3725,7 +3904,7 @@
         <v>90</v>
       </c>
       <c r="AK12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AL12" s="28" t="s">
         <v>69</v>
@@ -3734,7 +3913,6 @@
         <v>92</v>
       </c>
       <c r="AN12" s="29">
-        <f ca="1"/>
         <v>91076330092</v>
       </c>
       <c r="AO12" s="14" t="s">
@@ -3746,9 +3924,9 @@
       <c r="AQ12" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR12" s="19" t="str">
+      <c r="AR12" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS12" t="s">
         <v>96</v>
@@ -3802,10 +3980,10 @@
         <v>107</v>
       </c>
       <c r="BJ12" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK12" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK12" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL12" s="31" t="s">
         <v>110</v>
@@ -3820,12 +3998,12 @@
         <v>113</v>
       </c>
       <c r="BP12" s="38" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>193</v>
-      </c>
-    </row>
-    <row r="13" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>194</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="13" t="s">
@@ -3838,10 +4016,10 @@
         <v>70</v>
       </c>
       <c r="G13" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="H13" s="17" t="s">
         <v>195</v>
-      </c>
-      <c r="H13" s="17" t="s">
-        <v>196</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
@@ -3853,7 +4031,7 @@
         <v>74</v>
       </c>
       <c r="L13" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M13" s="14" t="s">
@@ -3887,7 +4065,7 @@
         <v>74</v>
       </c>
       <c r="W13" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X13" s="18" t="s">
@@ -3897,10 +4075,10 @@
         <v>81</v>
       </c>
       <c r="Z13" s="36" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AB13" s="37" t="s">
         <v>84</v>
@@ -3921,7 +4099,7 @@
         <v>87</v>
       </c>
       <c r="AH13" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46087</v>
       </c>
       <c r="AI13" s="18" t="s">
@@ -3931,7 +4109,7 @@
         <v>90</v>
       </c>
       <c r="AK13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AL13" s="28" t="s">
         <v>69</v>
@@ -3940,20 +4118,19 @@
         <v>92</v>
       </c>
       <c r="AN13" s="29">
-        <f ca="1"/>
         <v>12772211778</v>
       </c>
       <c r="AO13" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP13" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AQ13" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR13" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46087</v>
       </c>
       <c r="AS13" t="s">
@@ -3984,10 +4161,10 @@
         <v>69</v>
       </c>
       <c r="BB13" t="s">
+        <v>198</v>
+      </c>
+      <c r="BC13" s="34" t="s">
         <v>199</v>
-      </c>
-      <c r="BC13" s="34" t="s">
-        <v>200</v>
       </c>
       <c r="BD13" s="14" t="s">
         <v>102</v>
@@ -4008,10 +4185,10 @@
         <v>107</v>
       </c>
       <c r="BJ13" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK13" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK13" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL13" s="31" t="s">
         <v>110</v>
@@ -4029,9 +4206,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="13" t="s">
@@ -4044,10 +4221,10 @@
         <v>70</v>
       </c>
       <c r="G14" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="H14" s="17" t="s">
         <v>202</v>
-      </c>
-      <c r="H14" s="17" t="s">
-        <v>203</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
@@ -4059,7 +4236,7 @@
         <v>74</v>
       </c>
       <c r="L14" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M14" s="14" t="s">
@@ -4093,7 +4270,7 @@
         <v>74</v>
       </c>
       <c r="W14" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X14" s="18" t="s">
@@ -4106,10 +4283,10 @@
         <v>82</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="AB14" s="37" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AC14" s="1" t="s">
         <v>85</v>
@@ -4136,7 +4313,7 @@
         <v>90</v>
       </c>
       <c r="AK14" s="38" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AL14" s="28" t="s">
         <v>69</v>
@@ -4145,7 +4322,6 @@
         <v>92</v>
       </c>
       <c r="AN14" s="29">
-        <f ca="1"/>
         <v>61588847689</v>
       </c>
       <c r="AO14" s="14" t="s">
@@ -4157,9 +4333,9 @@
       <c r="AQ14" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR14" s="19" t="str">
+      <c r="AR14" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS14" t="s">
         <v>96</v>
@@ -4213,10 +4389,10 @@
         <v>107</v>
       </c>
       <c r="BJ14" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK14" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK14" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL14" s="31" t="s">
         <v>110</v>
@@ -4231,12 +4407,12 @@
         <v>113</v>
       </c>
       <c r="BP14" s="38" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="15" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>206</v>
-      </c>
-    </row>
-    <row r="15" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>207</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13" t="s">
@@ -4249,10 +4425,10 @@
         <v>70</v>
       </c>
       <c r="G15" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="H15" s="17" t="s">
         <v>208</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>209</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
@@ -4264,7 +4440,7 @@
         <v>74</v>
       </c>
       <c r="L15" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M15" s="14" t="s">
@@ -4298,7 +4474,7 @@
         <v>74</v>
       </c>
       <c r="W15" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X15" s="18" t="s">
@@ -4308,13 +4484,13 @@
         <v>81</v>
       </c>
       <c r="Z15" s="36" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AA15" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="AB15" s="37" t="s">
         <v>135</v>
-      </c>
-      <c r="AB15" s="37" t="s">
-        <v>136</v>
       </c>
       <c r="AC15" s="1" t="s">
         <v>85</v>
@@ -4332,7 +4508,7 @@
         <v>87</v>
       </c>
       <c r="AH15" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46087</v>
       </c>
       <c r="AI15" s="18" t="s">
@@ -4342,7 +4518,7 @@
         <v>90</v>
       </c>
       <c r="AK15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AL15" s="28" t="s">
         <v>69</v>
@@ -4351,20 +4527,19 @@
         <v>92</v>
       </c>
       <c r="AN15" s="29">
-        <f ca="1"/>
         <v>62719197684</v>
       </c>
       <c r="AO15" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP15" s="20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AQ15" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR15" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46087</v>
       </c>
       <c r="AS15" t="s">
@@ -4395,10 +4570,10 @@
         <v>69</v>
       </c>
       <c r="BB15" t="s">
+        <v>209</v>
+      </c>
+      <c r="BC15" t="s">
         <v>210</v>
-      </c>
-      <c r="BC15" t="s">
-        <v>211</v>
       </c>
       <c r="BD15" s="14" t="s">
         <v>102</v>
@@ -4419,10 +4594,10 @@
         <v>107</v>
       </c>
       <c r="BJ15" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK15" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK15" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL15" s="31" t="s">
         <v>110</v>
@@ -4437,16 +4612,16 @@
         <v>113</v>
       </c>
       <c r="BP15" s="33" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
-    <row r="16" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>69</v>
@@ -4455,10 +4630,10 @@
         <v>70</v>
       </c>
       <c r="G16" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="H16" s="17" t="s">
         <v>213</v>
-      </c>
-      <c r="H16" s="17" t="s">
-        <v>214</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
@@ -4470,7 +4645,7 @@
         <v>74</v>
       </c>
       <c r="L16" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45691</v>
       </c>
       <c r="M16" s="14" t="s">
@@ -4504,20 +4679,20 @@
         <v>74</v>
       </c>
       <c r="W16" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45691</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="Z16" s="38" t="s">
         <v>82</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AB16" s="37" t="s">
         <v>84</v>
@@ -4544,7 +4719,7 @@
         <v>89</v>
       </c>
       <c r="AJ16" s="18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AK16" s="1">
         <v>251</v>
@@ -4556,7 +4731,6 @@
         <v>92</v>
       </c>
       <c r="AN16" s="29">
-        <f ca="1"/>
         <v>28598841032</v>
       </c>
       <c r="AO16" s="14" t="s">
@@ -4568,9 +4742,9 @@
       <c r="AQ16" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR16" s="19" t="str">
+      <c r="AR16" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS16" t="s">
         <v>96</v>
@@ -4624,10 +4798,10 @@
         <v>107</v>
       </c>
       <c r="BJ16" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="BK16" s="31" t="s">
         <v>130</v>
-      </c>
-      <c r="BK16" s="31" t="s">
-        <v>131</v>
       </c>
       <c r="BL16" s="31" t="s">
         <v>110</v>
@@ -4646,33 +4820,69 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ10:AQ16 X10:X16 V10:V16 S10:S16 K10:K16 BI10:BI16 AX10:AX16" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ10:AQ16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ16 X2:X16 V2:V16 S2:S16 K2:K16 BI2:BI16 AX2:AX16" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX10:AX16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI10:BI16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K10:K16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S10:S16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X10:X16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="U4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="U5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="U6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="U7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="U8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="U9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="U10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="U11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="U12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="U13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="U14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="U15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="U2" r:id="rId1"/>
+    <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U4" r:id="rId3"/>
+    <hyperlink ref="U5" r:id="rId4"/>
+    <hyperlink ref="U6" r:id="rId5"/>
+    <hyperlink ref="U7" r:id="rId6"/>
+    <hyperlink ref="U8" r:id="rId7"/>
+    <hyperlink ref="U9" r:id="rId8"/>
+    <hyperlink ref="U10" r:id="rId9"/>
+    <hyperlink ref="U11" r:id="rId10"/>
+    <hyperlink ref="U12" r:id="rId11"/>
+    <hyperlink ref="U13" r:id="rId12"/>
+    <hyperlink ref="U14" r:id="rId13"/>
+    <hyperlink ref="U15" r:id="rId14"/>
+    <hyperlink ref="U16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
updated code after mergeing with Madhukar branch
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataBelgiumMKv01.xlsx
+++ b/Data/Hires/TestDataBelgiumMKv01.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="219">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -676,13 +676,19 @@
     <t>Test4</t>
   </si>
   <si>
-    <t>Tyrell</t>
-  </si>
-  <si>
-    <t>Pouros</t>
-  </si>
-  <si>
-    <t>Auto 80094408</t>
+    <t>10697920</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Louvenia</t>
+  </si>
+  <si>
+    <t>Bernhard</t>
+  </si>
+  <si>
+    <t>Auto 62715805</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -697,10 +703,13 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>Marty</t>
-  </si>
-  <si>
-    <t>Aufderhar</t>
+    <t>Test failed for 'Violette Medhurst' Employee: undefined&amp; find failed Screenshot Path:-&gt;H:\WorkdaySuite_Playwright_latestcode/WorkdayFailedScreenshot/2025-03-18T14-47-49-019Z.png</t>
+  </si>
+  <si>
+    <t>Violette</t>
+  </si>
+  <si>
+    <t>Medhurst</t>
   </si>
   <si>
     <t>Intern</t>
@@ -991,7 +1000,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -2370,7 +2379,12 @@
       <c r="A5" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C5" s="12"/>
+      <c r="B5" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>140</v>
+      </c>
       <c r="D5" s="13" t="s">
         <v>117</v>
       </c>
@@ -2381,10 +2395,10 @@
         <v>118</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I5" s="18">
         <v>25041111</v>
@@ -2437,13 +2451,13 @@
         <v>80</v>
       </c>
       <c r="Y5" s="24" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="Z5" t="s">
         <v>82</v>
       </c>
       <c r="AA5" s="25" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="AB5" t="s">
         <v>84</v>
@@ -2525,10 +2539,10 @@
         <v>69</v>
       </c>
       <c r="BB5" s="34" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="BC5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="BD5" s="14" t="s">
         <v>102</v>
@@ -2572,9 +2586,14 @@
     </row>
     <row r="6" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="12"/>
+        <v>147</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="D6" s="13" t="s">
         <v>68</v>
       </c>
@@ -2585,10 +2604,10 @@
         <v>70</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I6" s="18">
         <v>25041111</v>
@@ -2644,7 +2663,7 @@
         <v>81</v>
       </c>
       <c r="Z6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="AA6" s="25" t="s">
         <v>83</v>
@@ -2678,7 +2697,7 @@
         <v>90</v>
       </c>
       <c r="AK6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="AL6" s="28" t="s">
         <v>69</v>
@@ -2772,12 +2791,12 @@
         <v>113</v>
       </c>
       <c r="BP6" s="33" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13" t="s">
@@ -2790,10 +2809,10 @@
         <v>70</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I7" s="18">
         <v>25041111</v>
@@ -2846,13 +2865,13 @@
         <v>80</v>
       </c>
       <c r="Y7" s="24" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="Z7" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="AB7" s="37" t="s">
         <v>135</v>
@@ -2934,10 +2953,10 @@
         <v>69</v>
       </c>
       <c r="BB7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="BC7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="BD7" s="14" t="s">
         <v>102</v>
@@ -2976,12 +2995,12 @@
         <v>113</v>
       </c>
       <c r="BP7" s="33" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="13" t="s">
@@ -2994,10 +3013,10 @@
         <v>70</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
@@ -3050,13 +3069,13 @@
         <v>80</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="Z8" s="36" t="s">
         <v>122</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="AB8" s="37" t="s">
         <v>84</v>
@@ -3139,10 +3158,10 @@
         <v>69</v>
       </c>
       <c r="BB8" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="BC8" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="BD8" s="14" t="s">
         <v>102</v>
@@ -3186,7 +3205,7 @@
     </row>
     <row r="9" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13" t="s">
@@ -3199,10 +3218,10 @@
         <v>70</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
@@ -3255,13 +3274,13 @@
         <v>80</v>
       </c>
       <c r="Y9" s="24" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="Z9" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AB9" s="37" t="s">
         <v>135</v>
@@ -3343,10 +3362,10 @@
         <v>69</v>
       </c>
       <c r="BB9" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="BC9" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="BD9" s="14" t="s">
         <v>102</v>
@@ -3390,7 +3409,7 @@
     </row>
     <row r="10" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13" t="s">
@@ -3403,10 +3422,10 @@
         <v>70</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
@@ -3462,10 +3481,10 @@
         <v>81</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AB10" s="37" t="s">
         <v>135</v>
@@ -3474,7 +3493,7 @@
         <v>85</v>
       </c>
       <c r="AD10" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
@@ -3496,7 +3515,7 @@
         <v>90</v>
       </c>
       <c r="AK10" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AL10" s="28" t="s">
         <v>69</v>
@@ -3511,7 +3530,7 @@
         <v>93</v>
       </c>
       <c r="AP10" s="20" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AQ10" s="20" t="s">
         <v>95</v>
@@ -3590,12 +3609,12 @@
         <v>113</v>
       </c>
       <c r="BP10" s="38" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13" t="s">
@@ -3608,10 +3627,10 @@
         <v>70</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
@@ -3670,7 +3689,7 @@
         <v>82</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AB11" s="38" t="s">
         <v>84</v>
@@ -3700,7 +3719,7 @@
         <v>90</v>
       </c>
       <c r="AK11" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AL11" s="28" t="s">
         <v>69</v>
@@ -3752,10 +3771,10 @@
         <v>69</v>
       </c>
       <c r="BB11" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="BC11" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="BD11" s="14" t="s">
         <v>102</v>
@@ -3799,7 +3818,7 @@
     </row>
     <row r="12" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13" t="s">
@@ -3812,10 +3831,10 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
@@ -3874,7 +3893,7 @@
         <v>82</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="AB12" s="37" t="s">
         <v>135</v>
@@ -3904,7 +3923,7 @@
         <v>90</v>
       </c>
       <c r="AK12" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="AL12" s="28" t="s">
         <v>69</v>
@@ -3998,12 +4017,12 @@
         <v>113</v>
       </c>
       <c r="BP12" s="38" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="13" t="s">
@@ -4016,10 +4035,10 @@
         <v>70</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
@@ -4078,7 +4097,7 @@
         <v>122</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AB13" s="37" t="s">
         <v>84</v>
@@ -4109,7 +4128,7 @@
         <v>90</v>
       </c>
       <c r="AK13" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="AL13" s="28" t="s">
         <v>69</v>
@@ -4161,10 +4180,10 @@
         <v>69</v>
       </c>
       <c r="BB13" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="BD13" s="14" t="s">
         <v>102</v>
@@ -4208,7 +4227,7 @@
     </row>
     <row r="14" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="13" t="s">
@@ -4221,10 +4240,10 @@
         <v>70</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
@@ -4283,7 +4302,7 @@
         <v>82</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="AB14" s="37" t="s">
         <v>135</v>
@@ -4313,7 +4332,7 @@
         <v>90</v>
       </c>
       <c r="AK14" s="38" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="AL14" s="28" t="s">
         <v>69</v>
@@ -4407,12 +4426,12 @@
         <v>113</v>
       </c>
       <c r="BP14" s="38" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13" t="s">
@@ -4425,10 +4444,10 @@
         <v>70</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
@@ -4570,10 +4589,10 @@
         <v>69</v>
       </c>
       <c r="BB15" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="BC15" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="BD15" s="14" t="s">
         <v>102</v>
@@ -4612,12 +4631,12 @@
         <v>113</v>
       </c>
       <c r="BP15" s="33" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
@@ -4630,10 +4649,10 @@
         <v>70</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
@@ -4686,13 +4705,13 @@
         <v>80</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Z16" s="38" t="s">
         <v>82</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="AB16" s="37" t="s">
         <v>84</v>

</xml_diff>

<commit_message>
latest code for Slovenia and its working fine
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataBelgiumMKv01.xlsx
+++ b/Data/Hires/TestDataBelgiumMKv01.xlsx
@@ -1,20 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{0A4A3FDA-3E1F-48EE-B063-38BBD513C0E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="221">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -724,13 +739,19 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>Korey</t>
-  </si>
-  <si>
-    <t>Harber</t>
-  </si>
-  <si>
-    <t>Auto 39518004</t>
+    <t xml:space="preserve">Test failed for 'Angelita Grimes' Employee:{10697923}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByRole('button', { name: 'Approve' })[22m
+</t>
+  </si>
+  <si>
+    <t>Angelita</t>
+  </si>
+  <si>
+    <t>Grimes</t>
+  </si>
+  <si>
+    <t>Auto 3800979</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -766,13 +787,426 @@
     <t>Test8</t>
   </si>
   <si>
-    <t>Kattie</t>
-  </si>
-  <si>
-    <t>Olson</t>
-  </si>
-  <si>
-    <t>Auto 38867577</t>
+    <t xml:space="preserve">Test failed for 'Elinor Cruickshank' Employee:{10697931}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for locator('xpath=(//*[@data-automation-id=\'pex-search-result-header\']//a[contains(text(),\'10697931\')])[1]')[22m
+[2m  -   locator resolved to &lt;a data-uxi-rank="0" class="pexsearch-11mf54b" data…&gt;Elinor Cruickshank (10697931)&lt;/a&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #1[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #2[22m
+[2m  -   waiting 20ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #3[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #4[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #5[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #6[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #7[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #8[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #9[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #10[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #11[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #12[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #13[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #14[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #15[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #16[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #17[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #18[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #19[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #20[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #21[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #22[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #23[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #24[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #25[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #26[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #27[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #28[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #29[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #30[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #31[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #32[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #33[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #34[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #35[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #36[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #37[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #38[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #39[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #40[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #41[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #42[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #43[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #44[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #45[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #46[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #47[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #48[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #49[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #50[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #51[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #52[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #53[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #54[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #55[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #56[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; intercepts pointer events[22m
+[2m  - retrying click action, attempt #57[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-uxi-widget-type="popup" data-uxi-popup-type…&gt;…&lt;/div&gt; from &lt;div role="dialog" aria-modal="true" data-popup-versi…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #58[22m
+[2m  -   waiting 500ms[22m
+</t>
+  </si>
+  <si>
+    <t>Elinor</t>
+  </si>
+  <si>
+    <t>Cruickshank</t>
+  </si>
+  <si>
+    <t>Auto 23053516</t>
   </si>
   <si>
     <t>Visual Merchandising Manager_NEW</t>
@@ -919,58 +1353,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF4A4A4A"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="6"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
       <family val="3"/>
-      <sz val="6"/>
-      <name val="Courier New"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF800000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
@@ -982,25 +1416,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999938962981048"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -1019,8 +1453,12 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1030,15 +1468,25 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1049,14 +1497,22 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1071,17 +1527,29 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1473,9 +1941,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BP16"/>
-  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1545,7 +2013,7 @@
     <col min="68" max="68" width="16.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5" customHeight="1" spans="1:68" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="1" spans="1:68" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1751,7 +2219,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>65</v>
       </c>
@@ -1786,8 +2254,8 @@
         <v>74</v>
       </c>
       <c r="L2" s="19">
-        <f t="shared" ref="L2" si="0">TODAY()-31</f>
-        <v>45691</v>
+        <f t="shared" ref="L2" ca="1" si="0">TODAY()-31</f>
+        <v>45704</v>
       </c>
       <c r="M2" s="14" t="s">
         <v>69</v>
@@ -1820,8 +2288,8 @@
         <v>74</v>
       </c>
       <c r="W2" s="23">
-        <f t="shared" ref="W2" si="1">L2</f>
-        <v>45691</v>
+        <f t="shared" ref="W2" ca="1" si="1">L2</f>
+        <v>45704</v>
       </c>
       <c r="X2" s="18" t="s">
         <v>80</v>
@@ -1872,8 +2340,8 @@
         <v>92</v>
       </c>
       <c r="AN2" s="29">
-        <f t="array" ref="AN2:AN16">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
-        <v>52464079638</v>
+        <f t="array" aca="1" ref="AN2:AN16" ca="1">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
+        <v>74415766585</v>
       </c>
       <c r="AO2" s="14" t="s">
         <v>93</v>
@@ -1884,9 +2352,9 @@
       <c r="AQ2" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR2" s="19">
+      <c r="AR2" s="19" t="str">
         <f>AH2</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS2" t="s">
         <v>96</v>
@@ -1961,7 +2429,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="3" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>115</v>
       </c>
@@ -1996,8 +2464,8 @@
         <v>74</v>
       </c>
       <c r="L3" s="19">
-        <f t="shared" ref="L3:L16" si="2">TODAY()-31</f>
-        <v>45691</v>
+        <f t="shared" ref="L3:L16" ca="1" si="2">TODAY()-31</f>
+        <v>45704</v>
       </c>
       <c r="M3" s="14" t="s">
         <v>69</v>
@@ -2030,8 +2498,8 @@
         <v>74</v>
       </c>
       <c r="W3" s="23">
-        <f t="shared" ref="W3:W16" si="3">L3</f>
-        <v>45691</v>
+        <f t="shared" ref="W3:W16" ca="1" si="3">L3</f>
+        <v>45704</v>
       </c>
       <c r="X3" s="18" t="s">
         <v>80</v>
@@ -2064,8 +2532,8 @@
         <v>87</v>
       </c>
       <c r="AH3" s="19">
-        <f>TODAY()+365</f>
-        <v>46087</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46100</v>
       </c>
       <c r="AI3" s="18" t="s">
         <v>89</v>
@@ -2083,7 +2551,8 @@
         <v>92</v>
       </c>
       <c r="AN3" s="29">
-        <v>81569448446</v>
+        <f ca="1"/>
+        <v>64966629264</v>
       </c>
       <c r="AO3" s="14" t="s">
         <v>93</v>
@@ -2095,8 +2564,8 @@
         <v>95</v>
       </c>
       <c r="AR3" s="19">
-        <f t="shared" ref="AR3:AR16" si="4">AH3</f>
-        <v>46087</v>
+        <f t="shared" ref="AR3:AR16" ca="1" si="4">AH3</f>
+        <v>46100</v>
       </c>
       <c r="AS3" t="s">
         <v>126</v>
@@ -2171,7 +2640,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>131</v>
       </c>
@@ -2201,8 +2670,8 @@
         <v>74</v>
       </c>
       <c r="L4" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M4" s="14" t="s">
         <v>69</v>
@@ -2235,8 +2704,8 @@
         <v>74</v>
       </c>
       <c r="W4" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X4" s="18" t="s">
         <v>80</v>
@@ -2287,7 +2756,8 @@
         <v>92</v>
       </c>
       <c r="AN4" s="29">
-        <v>19431753549</v>
+        <f ca="1"/>
+        <v>95182528772</v>
       </c>
       <c r="AO4" s="14" t="s">
         <v>93</v>
@@ -2298,9 +2768,9 @@
       <c r="AQ4" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR4" s="19">
+      <c r="AR4" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS4" t="s">
         <v>96</v>
@@ -2375,7 +2845,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="5" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>138</v>
       </c>
@@ -2410,8 +2880,8 @@
         <v>74</v>
       </c>
       <c r="L5" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M5" s="14" t="s">
         <v>69</v>
@@ -2444,8 +2914,8 @@
         <v>74</v>
       </c>
       <c r="W5" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X5" s="18" t="s">
         <v>80</v>
@@ -2496,7 +2966,8 @@
         <v>92</v>
       </c>
       <c r="AN5" s="29">
-        <v>91305818781</v>
+        <f ca="1"/>
+        <v>28666154230</v>
       </c>
       <c r="AO5" s="14" t="s">
         <v>93</v>
@@ -2507,9 +2978,9 @@
       <c r="AQ5" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR5" s="19">
+      <c r="AR5" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS5" t="s">
         <v>126</v>
@@ -2584,7 +3055,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>147</v>
       </c>
@@ -2619,8 +3090,8 @@
         <v>74</v>
       </c>
       <c r="L6" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M6" s="14" t="s">
         <v>69</v>
@@ -2653,8 +3124,8 @@
         <v>74</v>
       </c>
       <c r="W6" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X6" s="18" t="s">
         <v>80</v>
@@ -2687,8 +3158,8 @@
         <v>87</v>
       </c>
       <c r="AH6" s="19">
-        <f>TODAY()+365</f>
-        <v>46087</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46100</v>
       </c>
       <c r="AI6" s="18" t="s">
         <v>89</v>
@@ -2706,7 +3177,8 @@
         <v>92</v>
       </c>
       <c r="AN6" s="29">
-        <v>28307817987</v>
+        <f ca="1"/>
+        <v>27176082664</v>
       </c>
       <c r="AO6" s="14" t="s">
         <v>93</v>
@@ -2718,8 +3190,8 @@
         <v>95</v>
       </c>
       <c r="AR6" s="19">
-        <f t="shared" si="4"/>
-        <v>46087</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46100</v>
       </c>
       <c r="AS6" t="s">
         <v>96</v>
@@ -2794,11 +3266,16 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C7" s="12"/>
+      <c r="B7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="D7" s="13" t="s">
         <v>117</v>
       </c>
@@ -2809,10 +3286,10 @@
         <v>70</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I7" s="18">
         <v>25041111</v>
@@ -2824,8 +3301,8 @@
         <v>74</v>
       </c>
       <c r="L7" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M7" s="14" t="s">
         <v>69</v>
@@ -2858,20 +3335,20 @@
         <v>74</v>
       </c>
       <c r="W7" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X7" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y7" s="24" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Z7" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA7" s="25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AB7" s="37" t="s">
         <v>135</v>
@@ -2910,7 +3387,8 @@
         <v>92</v>
       </c>
       <c r="AN7" s="29">
-        <v>90116436576</v>
+        <f ca="1"/>
+        <v>60539593966</v>
       </c>
       <c r="AO7" s="14" t="s">
         <v>93</v>
@@ -2921,9 +3399,9 @@
       <c r="AQ7" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR7" s="19">
+      <c r="AR7" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS7" t="s">
         <v>96</v>
@@ -2953,10 +3431,10 @@
         <v>69</v>
       </c>
       <c r="BB7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="BC7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="BD7" s="14" t="s">
         <v>102</v>
@@ -2998,9 +3476,9 @@
         <v>153</v>
       </c>
     </row>
-    <row r="8" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="13" t="s">
@@ -3013,10 +3491,10 @@
         <v>70</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
@@ -3028,8 +3506,8 @@
         <v>74</v>
       </c>
       <c r="L8" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M8" s="14" t="s">
         <v>69</v>
@@ -3062,20 +3540,20 @@
         <v>74</v>
       </c>
       <c r="W8" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X8" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Z8" s="36" t="s">
         <v>122</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AB8" s="37" t="s">
         <v>84</v>
@@ -3096,8 +3574,8 @@
         <v>87</v>
       </c>
       <c r="AH8" s="19">
-        <f>TODAY()+365</f>
-        <v>46087</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46100</v>
       </c>
       <c r="AI8" s="18" t="s">
         <v>89</v>
@@ -3115,7 +3593,8 @@
         <v>92</v>
       </c>
       <c r="AN8" s="29">
-        <v>88397911747</v>
+        <f ca="1"/>
+        <v>58481955591</v>
       </c>
       <c r="AO8" s="14" t="s">
         <v>93</v>
@@ -3127,8 +3606,8 @@
         <v>95</v>
       </c>
       <c r="AR8" s="19">
-        <f t="shared" si="4"/>
-        <v>46087</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46100</v>
       </c>
       <c r="AS8" t="s">
         <v>96</v>
@@ -3158,10 +3637,10 @@
         <v>69</v>
       </c>
       <c r="BB8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="BC8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="BD8" s="14" t="s">
         <v>102</v>
@@ -3203,11 +3682,16 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C9" s="12"/>
+        <v>169</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="D9" s="13" t="s">
         <v>117</v>
       </c>
@@ -3218,10 +3702,10 @@
         <v>70</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
@@ -3233,8 +3717,8 @@
         <v>74</v>
       </c>
       <c r="L9" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M9" s="14" t="s">
         <v>69</v>
@@ -3267,20 +3751,20 @@
         <v>74</v>
       </c>
       <c r="W9" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X9" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y9" s="24" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="Z9" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="AB9" s="37" t="s">
         <v>135</v>
@@ -3319,7 +3803,8 @@
         <v>92</v>
       </c>
       <c r="AN9" s="29">
-        <v>57149063321</v>
+        <f ca="1"/>
+        <v>59981468405</v>
       </c>
       <c r="AO9" s="14" t="s">
         <v>93</v>
@@ -3330,9 +3815,9 @@
       <c r="AQ9" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR9" s="19">
+      <c r="AR9" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS9" t="s">
         <v>96</v>
@@ -3362,10 +3847,10 @@
         <v>69</v>
       </c>
       <c r="BB9" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="BC9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="BD9" s="14" t="s">
         <v>102</v>
@@ -3407,9 +3892,9 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13" t="s">
@@ -3422,10 +3907,10 @@
         <v>70</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
@@ -3437,8 +3922,8 @@
         <v>74</v>
       </c>
       <c r="L10" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M10" s="14" t="s">
         <v>69</v>
@@ -3471,8 +3956,8 @@
         <v>74</v>
       </c>
       <c r="W10" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X10" s="18" t="s">
         <v>80</v>
@@ -3481,10 +3966,10 @@
         <v>81</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AB10" s="37" t="s">
         <v>135</v>
@@ -3493,7 +3978,7 @@
         <v>85</v>
       </c>
       <c r="AD10" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
@@ -3505,8 +3990,8 @@
         <v>87</v>
       </c>
       <c r="AH10" s="19">
-        <f>TODAY()+365</f>
-        <v>46087</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46100</v>
       </c>
       <c r="AI10" s="18" t="s">
         <v>89</v>
@@ -3515,7 +4000,7 @@
         <v>90</v>
       </c>
       <c r="AK10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AL10" s="28" t="s">
         <v>69</v>
@@ -3524,20 +4009,21 @@
         <v>92</v>
       </c>
       <c r="AN10" s="29">
-        <v>74848109800</v>
+        <f ca="1"/>
+        <v>77615119087</v>
       </c>
       <c r="AO10" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP10" s="20" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AQ10" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR10" s="19">
-        <f t="shared" si="4"/>
-        <v>46087</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46100</v>
       </c>
       <c r="AS10" t="s">
         <v>96</v>
@@ -3609,12 +4095,12 @@
         <v>113</v>
       </c>
       <c r="BP10" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
-    <row r="11" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13" t="s">
@@ -3627,10 +4113,10 @@
         <v>70</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
@@ -3642,8 +4128,8 @@
         <v>74</v>
       </c>
       <c r="L11" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M11" s="14" t="s">
         <v>69</v>
@@ -3676,8 +4162,8 @@
         <v>74</v>
       </c>
       <c r="W11" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X11" s="18" t="s">
         <v>80</v>
@@ -3689,7 +4175,7 @@
         <v>82</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AB11" s="38" t="s">
         <v>84</v>
@@ -3719,7 +4205,7 @@
         <v>90</v>
       </c>
       <c r="AK11" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="AL11" s="28" t="s">
         <v>69</v>
@@ -3728,7 +4214,8 @@
         <v>92</v>
       </c>
       <c r="AN11" s="29">
-        <v>83735190113</v>
+        <f ca="1"/>
+        <v>65017546092</v>
       </c>
       <c r="AO11" s="14" t="s">
         <v>93</v>
@@ -3739,9 +4226,9 @@
       <c r="AQ11" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR11" s="19">
+      <c r="AR11" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS11" t="s">
         <v>96</v>
@@ -3771,10 +4258,10 @@
         <v>69</v>
       </c>
       <c r="BB11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BC11" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="BD11" s="14" t="s">
         <v>102</v>
@@ -3816,9 +4303,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13" t="s">
@@ -3831,10 +4318,10 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
@@ -3846,8 +4333,8 @@
         <v>74</v>
       </c>
       <c r="L12" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M12" s="14" t="s">
         <v>69</v>
@@ -3880,8 +4367,8 @@
         <v>74</v>
       </c>
       <c r="W12" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X12" s="18" t="s">
         <v>80</v>
@@ -3893,7 +4380,7 @@
         <v>82</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="AB12" s="37" t="s">
         <v>135</v>
@@ -3923,7 +4410,7 @@
         <v>90</v>
       </c>
       <c r="AK12" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="AL12" s="28" t="s">
         <v>69</v>
@@ -3932,7 +4419,8 @@
         <v>92</v>
       </c>
       <c r="AN12" s="29">
-        <v>91076330092</v>
+        <f ca="1"/>
+        <v>69463381017</v>
       </c>
       <c r="AO12" s="14" t="s">
         <v>93</v>
@@ -3943,9 +4431,9 @@
       <c r="AQ12" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR12" s="19">
+      <c r="AR12" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS12" t="s">
         <v>96</v>
@@ -4017,12 +4505,12 @@
         <v>113</v>
       </c>
       <c r="BP12" s="38" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
-    <row r="13" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="13" t="s">
@@ -4035,10 +4523,10 @@
         <v>70</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
@@ -4050,8 +4538,8 @@
         <v>74</v>
       </c>
       <c r="L13" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M13" s="14" t="s">
         <v>69</v>
@@ -4084,8 +4572,8 @@
         <v>74</v>
       </c>
       <c r="W13" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X13" s="18" t="s">
         <v>80</v>
@@ -4097,7 +4585,7 @@
         <v>122</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="AB13" s="37" t="s">
         <v>84</v>
@@ -4118,8 +4606,8 @@
         <v>87</v>
       </c>
       <c r="AH13" s="19">
-        <f>TODAY()+365</f>
-        <v>46087</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46100</v>
       </c>
       <c r="AI13" s="18" t="s">
         <v>89</v>
@@ -4128,7 +4616,7 @@
         <v>90</v>
       </c>
       <c r="AK13" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="AL13" s="28" t="s">
         <v>69</v>
@@ -4137,7 +4625,8 @@
         <v>92</v>
       </c>
       <c r="AN13" s="29">
-        <v>12772211778</v>
+        <f ca="1"/>
+        <v>68204494491</v>
       </c>
       <c r="AO13" s="14" t="s">
         <v>93</v>
@@ -4149,8 +4638,8 @@
         <v>95</v>
       </c>
       <c r="AR13" s="19">
-        <f t="shared" si="4"/>
-        <v>46087</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46100</v>
       </c>
       <c r="AS13" t="s">
         <v>96</v>
@@ -4180,10 +4669,10 @@
         <v>69</v>
       </c>
       <c r="BB13" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="BD13" s="14" t="s">
         <v>102</v>
@@ -4225,9 +4714,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="13" t="s">
@@ -4240,10 +4729,10 @@
         <v>70</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
@@ -4255,8 +4744,8 @@
         <v>74</v>
       </c>
       <c r="L14" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M14" s="14" t="s">
         <v>69</v>
@@ -4289,8 +4778,8 @@
         <v>74</v>
       </c>
       <c r="W14" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X14" s="18" t="s">
         <v>80</v>
@@ -4302,7 +4791,7 @@
         <v>82</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="AB14" s="37" t="s">
         <v>135</v>
@@ -4332,7 +4821,7 @@
         <v>90</v>
       </c>
       <c r="AK14" s="38" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="AL14" s="28" t="s">
         <v>69</v>
@@ -4341,7 +4830,8 @@
         <v>92</v>
       </c>
       <c r="AN14" s="29">
-        <v>61588847689</v>
+        <f ca="1"/>
+        <v>24226361657</v>
       </c>
       <c r="AO14" s="14" t="s">
         <v>93</v>
@@ -4352,9 +4842,9 @@
       <c r="AQ14" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR14" s="19">
+      <c r="AR14" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS14" t="s">
         <v>96</v>
@@ -4426,12 +4916,12 @@
         <v>113</v>
       </c>
       <c r="BP14" s="38" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
-    <row r="15" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13" t="s">
@@ -4444,10 +4934,10 @@
         <v>70</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
@@ -4459,8 +4949,8 @@
         <v>74</v>
       </c>
       <c r="L15" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M15" s="14" t="s">
         <v>69</v>
@@ -4493,8 +4983,8 @@
         <v>74</v>
       </c>
       <c r="W15" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X15" s="18" t="s">
         <v>80</v>
@@ -4527,8 +5017,8 @@
         <v>87</v>
       </c>
       <c r="AH15" s="19">
-        <f>TODAY()+365</f>
-        <v>46087</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46100</v>
       </c>
       <c r="AI15" s="18" t="s">
         <v>89</v>
@@ -4546,7 +5036,8 @@
         <v>92</v>
       </c>
       <c r="AN15" s="29">
-        <v>62719197684</v>
+        <f ca="1"/>
+        <v>75635122197</v>
       </c>
       <c r="AO15" s="14" t="s">
         <v>93</v>
@@ -4558,8 +5049,8 @@
         <v>95</v>
       </c>
       <c r="AR15" s="19">
-        <f t="shared" si="4"/>
-        <v>46087</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46100</v>
       </c>
       <c r="AS15" t="s">
         <v>96</v>
@@ -4589,10 +5080,10 @@
         <v>69</v>
       </c>
       <c r="BB15" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="BC15" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="BD15" s="14" t="s">
         <v>102</v>
@@ -4634,9 +5125,9 @@
         <v>153</v>
       </c>
     </row>
-    <row r="16" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
@@ -4649,10 +5140,10 @@
         <v>70</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
@@ -4664,8 +5155,8 @@
         <v>74</v>
       </c>
       <c r="L16" s="19">
-        <f t="shared" si="2"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45704</v>
       </c>
       <c r="M16" s="14" t="s">
         <v>69</v>
@@ -4698,20 +5189,20 @@
         <v>74</v>
       </c>
       <c r="W16" s="23">
-        <f t="shared" si="3"/>
-        <v>45691</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45704</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="Z16" s="38" t="s">
         <v>82</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="AB16" s="37" t="s">
         <v>84</v>
@@ -4750,7 +5241,8 @@
         <v>92</v>
       </c>
       <c r="AN16" s="29">
-        <v>28598841032</v>
+        <f ca="1"/>
+        <v>21045840423</v>
       </c>
       <c r="AO16" s="14" t="s">
         <v>93</v>
@@ -4761,9 +5253,9 @@
       <c r="AQ16" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR16" s="19">
+      <c r="AR16" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AS16" t="s">
         <v>96</v>
@@ -4839,69 +5331,33 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="14">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ10:AQ16">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ10:AQ16 X10:X16 V10:V16 S10:S16 K10:K16 BI10:BI16 AX10:AX16" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX10:AX16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI10:BI16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K10:K16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S10:S16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X10:X16">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ16 X2:X16 V2:V16 S2:S16 K2:K16 BI2:BI16 AX2:AX16" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1"/>
-    <hyperlink ref="U3" r:id="rId2"/>
-    <hyperlink ref="U4" r:id="rId3"/>
-    <hyperlink ref="U5" r:id="rId4"/>
-    <hyperlink ref="U6" r:id="rId5"/>
-    <hyperlink ref="U7" r:id="rId6"/>
-    <hyperlink ref="U8" r:id="rId7"/>
-    <hyperlink ref="U9" r:id="rId8"/>
-    <hyperlink ref="U10" r:id="rId9"/>
-    <hyperlink ref="U11" r:id="rId10"/>
-    <hyperlink ref="U12" r:id="rId11"/>
-    <hyperlink ref="U13" r:id="rId12"/>
-    <hyperlink ref="U14" r:id="rId13"/>
-    <hyperlink ref="U15" r:id="rId14"/>
-    <hyperlink ref="U16" r:id="rId15"/>
+    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="U4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="U5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="U6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="U7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="U8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="U9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="U10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="U11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="U12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="U13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="U14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="U15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Code has been updated for Hungary
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataBelgiumMKv01.xlsx
+++ b/Data/Hires/TestDataBelgiumMKv01.xlsx
@@ -1,35 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{0A4A3FDA-3E1F-48EE-B063-38BBD513C0E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="222">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -739,19 +724,19 @@
     <t>Test6</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Angelita Grimes' Employee:{10697923}TimeoutError: locator.click: Timeout 30000ms exceeded.
+    <t xml:space="preserve">Test failed for 'Katelin Emmerich-Moen' Employee:{undefined}TimeoutError: locator.click: Timeout 30000ms exceeded.
 Call log:
-  [2m- waiting for getByRole('button', { name: 'Approve' })[22m
+  [2m- waiting for getByRole('button', { name: 'Personal Information Change: Katelin Emmerich-Moen' }).first()[22m
 </t>
   </si>
   <si>
-    <t>Angelita</t>
-  </si>
-  <si>
-    <t>Grimes</t>
-  </si>
-  <si>
-    <t>Auto 3800979</t>
+    <t>Katelin</t>
+  </si>
+  <si>
+    <t>Emmerich-Moen</t>
+  </si>
+  <si>
+    <t>Auto 8194915</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -766,13 +751,384 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>Melissa</t>
-  </si>
-  <si>
-    <t>Yundt</t>
-  </si>
-  <si>
-    <t>Auto 51742445</t>
+    <t xml:space="preserve">Test failed for 'Rosamond Purdy' Employee:{undefined}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for locator('xpath=(//*[@data-automation-label=\'Fixed Term (Fixed Term)\' or text()=\'Fixed Term (Fixed Term)\'])[1]')[22m
+[2m  -   locator resolved to &lt;div class="gwt-Label WOPO WHOO" id="promptOption-gwt…&gt;Fixed Term (Fixed Term)&lt;/div&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #1[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #2[22m
+[2m  -   waiting 20ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #3[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #4[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #5[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #6[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #7[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #8[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #9[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #10[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #11[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #12[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #13[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #14[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #15[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #16[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #17[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #18[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #19[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #20[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #21[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #22[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #23[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #24[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #25[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #26[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #27[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #28[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #29[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #30[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #31[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #32[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #33[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #34[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #35[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #36[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #37[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #38[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #39[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #40[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #41[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #42[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #43[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #44[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #45[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #46[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #47[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #48[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #49[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #50[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #51[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div data-automation-id="promptOption" data-automatio…&gt;More than 3 Months&lt;/div&gt; from &lt;div data-popup-type="ck" data-popup-version="2" clas…&gt;…&lt;/div&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #52[22m
+[2m  -   waiting 500ms[22m
+</t>
+  </si>
+  <si>
+    <t>Rosamond</t>
+  </si>
+  <si>
+    <t>Purdy</t>
+  </si>
+  <si>
+    <t>Auto 60996420</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -1353,58 +1709,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color indexed="8"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color indexed="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FF4A4A4A"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FF1F1F1F"/>
+      <family val="3"/>
       <sz val="6"/>
-      <color rgb="FF1F1F1F"/>
       <name val="Courier New"/>
-      <family val="3"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FF800000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1416,19 +1772,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1453,12 +1809,8 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -1468,25 +1820,15 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -1497,22 +1839,14 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left style="thin"/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -1527,29 +1861,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <left style="thin"/>
+      <right style="thin"/>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1941,9 +2263,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BP16"/>
-  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -2013,7 +2335,7 @@
     <col min="68" max="68" width="16.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.5" customHeight="1" spans="1:68" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2219,7 +2541,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>65</v>
       </c>
@@ -2254,7 +2576,7 @@
         <v>74</v>
       </c>
       <c r="L2" s="19">
-        <f t="shared" ref="L2" ca="1" si="0">TODAY()-31</f>
+        <f t="shared" ref="L2" si="0">TODAY()-31</f>
         <v>45704</v>
       </c>
       <c r="M2" s="14" t="s">
@@ -2288,7 +2610,7 @@
         <v>74</v>
       </c>
       <c r="W2" s="23">
-        <f t="shared" ref="W2" ca="1" si="1">L2</f>
+        <f t="shared" ref="W2" si="1">L2</f>
         <v>45704</v>
       </c>
       <c r="X2" s="18" t="s">
@@ -2340,7 +2662,7 @@
         <v>92</v>
       </c>
       <c r="AN2" s="29">
-        <f t="array" aca="1" ref="AN2:AN16" ca="1">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
+        <f t="array" ref="AN2:AN16">_xlfn.RANDARRAY(15,1,12345678901,99999999999,TRUE)</f>
         <v>74415766585</v>
       </c>
       <c r="AO2" s="14" t="s">
@@ -2352,9 +2674,9 @@
       <c r="AQ2" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR2" s="19" t="str">
+      <c r="AR2" s="19">
         <f>AH2</f>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS2" t="s">
         <v>96</v>
@@ -2429,7 +2751,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="3" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>115</v>
       </c>
@@ -2464,7 +2786,7 @@
         <v>74</v>
       </c>
       <c r="L3" s="19">
-        <f t="shared" ref="L3:L16" ca="1" si="2">TODAY()-31</f>
+        <f t="shared" ref="L3:L16" si="2">TODAY()-31</f>
         <v>45704</v>
       </c>
       <c r="M3" s="14" t="s">
@@ -2498,7 +2820,7 @@
         <v>74</v>
       </c>
       <c r="W3" s="23">
-        <f t="shared" ref="W3:W16" ca="1" si="3">L3</f>
+        <f t="shared" ref="W3:W16" si="3">L3</f>
         <v>45704</v>
       </c>
       <c r="X3" s="18" t="s">
@@ -2532,7 +2854,7 @@
         <v>87</v>
       </c>
       <c r="AH3" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46100</v>
       </c>
       <c r="AI3" s="18" t="s">
@@ -2551,7 +2873,6 @@
         <v>92</v>
       </c>
       <c r="AN3" s="29">
-        <f ca="1"/>
         <v>64966629264</v>
       </c>
       <c r="AO3" s="14" t="s">
@@ -2564,7 +2885,7 @@
         <v>95</v>
       </c>
       <c r="AR3" s="19">
-        <f t="shared" ref="AR3:AR16" ca="1" si="4">AH3</f>
+        <f t="shared" ref="AR3:AR16" si="4">AH3</f>
         <v>46100</v>
       </c>
       <c r="AS3" t="s">
@@ -2640,7 +2961,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>131</v>
       </c>
@@ -2670,7 +2991,7 @@
         <v>74</v>
       </c>
       <c r="L4" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M4" s="14" t="s">
@@ -2704,7 +3025,7 @@
         <v>74</v>
       </c>
       <c r="W4" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X4" s="18" t="s">
@@ -2756,7 +3077,6 @@
         <v>92</v>
       </c>
       <c r="AN4" s="29">
-        <f ca="1"/>
         <v>95182528772</v>
       </c>
       <c r="AO4" s="14" t="s">
@@ -2768,9 +3088,9 @@
       <c r="AQ4" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR4" s="19" t="str">
+      <c r="AR4" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS4" t="s">
         <v>96</v>
@@ -2845,7 +3165,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="5" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>138</v>
       </c>
@@ -2880,7 +3200,7 @@
         <v>74</v>
       </c>
       <c r="L5" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M5" s="14" t="s">
@@ -2914,7 +3234,7 @@
         <v>74</v>
       </c>
       <c r="W5" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X5" s="18" t="s">
@@ -2966,7 +3286,6 @@
         <v>92</v>
       </c>
       <c r="AN5" s="29">
-        <f ca="1"/>
         <v>28666154230</v>
       </c>
       <c r="AO5" s="14" t="s">
@@ -2978,9 +3297,9 @@
       <c r="AQ5" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR5" s="19" t="str">
+      <c r="AR5" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS5" t="s">
         <v>126</v>
@@ -3055,7 +3374,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>147</v>
       </c>
@@ -3090,7 +3409,7 @@
         <v>74</v>
       </c>
       <c r="L6" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M6" s="14" t="s">
@@ -3124,7 +3443,7 @@
         <v>74</v>
       </c>
       <c r="W6" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X6" s="18" t="s">
@@ -3158,7 +3477,7 @@
         <v>87</v>
       </c>
       <c r="AH6" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46100</v>
       </c>
       <c r="AI6" s="18" t="s">
@@ -3177,7 +3496,6 @@
         <v>92</v>
       </c>
       <c r="AN6" s="29">
-        <f ca="1"/>
         <v>27176082664</v>
       </c>
       <c r="AO6" s="14" t="s">
@@ -3190,7 +3508,7 @@
         <v>95</v>
       </c>
       <c r="AR6" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46100</v>
       </c>
       <c r="AS6" t="s">
@@ -3266,7 +3584,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>154</v>
       </c>
@@ -3301,7 +3619,7 @@
         <v>74</v>
       </c>
       <c r="L7" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M7" s="14" t="s">
@@ -3335,7 +3653,7 @@
         <v>74</v>
       </c>
       <c r="W7" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X7" s="18" t="s">
@@ -3387,7 +3705,6 @@
         <v>92</v>
       </c>
       <c r="AN7" s="29">
-        <f ca="1"/>
         <v>60539593966</v>
       </c>
       <c r="AO7" s="14" t="s">
@@ -3399,9 +3716,9 @@
       <c r="AQ7" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR7" s="19" t="str">
+      <c r="AR7" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS7" t="s">
         <v>96</v>
@@ -3476,11 +3793,16 @@
         <v>153</v>
       </c>
     </row>
-    <row r="8" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C8" s="12"/>
+      <c r="B8" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="D8" s="13" t="s">
         <v>117</v>
       </c>
@@ -3491,10 +3813,10 @@
         <v>70</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I8" s="18">
         <v>25041111</v>
@@ -3506,7 +3828,7 @@
         <v>74</v>
       </c>
       <c r="L8" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M8" s="14" t="s">
@@ -3540,20 +3862,20 @@
         <v>74</v>
       </c>
       <c r="W8" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X8" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Z8" s="36" t="s">
         <v>122</v>
       </c>
       <c r="AA8" s="25" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AB8" s="37" t="s">
         <v>84</v>
@@ -3574,7 +3896,7 @@
         <v>87</v>
       </c>
       <c r="AH8" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46100</v>
       </c>
       <c r="AI8" s="18" t="s">
@@ -3593,7 +3915,6 @@
         <v>92</v>
       </c>
       <c r="AN8" s="29">
-        <f ca="1"/>
         <v>58481955591</v>
       </c>
       <c r="AO8" s="14" t="s">
@@ -3606,7 +3927,7 @@
         <v>95</v>
       </c>
       <c r="AR8" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46100</v>
       </c>
       <c r="AS8" t="s">
@@ -3637,10 +3958,10 @@
         <v>69</v>
       </c>
       <c r="BB8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="BC8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="BD8" s="14" t="s">
         <v>102</v>
@@ -3682,12 +4003,12 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>67</v>
@@ -3702,10 +4023,10 @@
         <v>70</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I9" s="18">
         <v>25041111</v>
@@ -3717,7 +4038,7 @@
         <v>74</v>
       </c>
       <c r="L9" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M9" s="14" t="s">
@@ -3751,20 +4072,20 @@
         <v>74</v>
       </c>
       <c r="W9" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X9" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y9" s="24" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Z9" s="36" t="s">
         <v>82</v>
       </c>
       <c r="AA9" s="25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AB9" s="37" t="s">
         <v>135</v>
@@ -3803,7 +4124,6 @@
         <v>92</v>
       </c>
       <c r="AN9" s="29">
-        <f ca="1"/>
         <v>59981468405</v>
       </c>
       <c r="AO9" s="14" t="s">
@@ -3815,9 +4135,9 @@
       <c r="AQ9" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR9" s="19" t="str">
+      <c r="AR9" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS9" t="s">
         <v>96</v>
@@ -3847,10 +4167,10 @@
         <v>69</v>
       </c>
       <c r="BB9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="BC9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="BD9" s="14" t="s">
         <v>102</v>
@@ -3892,9 +4212,9 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13" t="s">
@@ -3907,10 +4227,10 @@
         <v>70</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I10" s="18">
         <v>25041111</v>
@@ -3922,7 +4242,7 @@
         <v>74</v>
       </c>
       <c r="L10" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M10" s="14" t="s">
@@ -3956,7 +4276,7 @@
         <v>74</v>
       </c>
       <c r="W10" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X10" s="18" t="s">
@@ -3966,10 +4286,10 @@
         <v>81</v>
       </c>
       <c r="Z10" s="36" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AA10" s="25" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AB10" s="37" t="s">
         <v>135</v>
@@ -3978,7 +4298,7 @@
         <v>85</v>
       </c>
       <c r="AD10" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AE10" s="26">
         <v>10</v>
@@ -3990,7 +4310,7 @@
         <v>87</v>
       </c>
       <c r="AH10" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46100</v>
       </c>
       <c r="AI10" s="18" t="s">
@@ -4000,7 +4320,7 @@
         <v>90</v>
       </c>
       <c r="AK10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AL10" s="28" t="s">
         <v>69</v>
@@ -4009,20 +4329,19 @@
         <v>92</v>
       </c>
       <c r="AN10" s="29">
-        <f ca="1"/>
         <v>77615119087</v>
       </c>
       <c r="AO10" s="14" t="s">
         <v>93</v>
       </c>
       <c r="AP10" s="20" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AQ10" s="20" t="s">
         <v>95</v>
       </c>
       <c r="AR10" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46100</v>
       </c>
       <c r="AS10" t="s">
@@ -4095,12 +4414,12 @@
         <v>113</v>
       </c>
       <c r="BP10" s="38" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
-    <row r="11" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13" t="s">
@@ -4113,10 +4432,10 @@
         <v>70</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I11" s="18">
         <v>25041111</v>
@@ -4128,7 +4447,7 @@
         <v>74</v>
       </c>
       <c r="L11" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M11" s="14" t="s">
@@ -4162,7 +4481,7 @@
         <v>74</v>
       </c>
       <c r="W11" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X11" s="18" t="s">
@@ -4175,7 +4494,7 @@
         <v>82</v>
       </c>
       <c r="AA11" s="25" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AB11" s="38" t="s">
         <v>84</v>
@@ -4205,7 +4524,7 @@
         <v>90</v>
       </c>
       <c r="AK11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="AL11" s="28" t="s">
         <v>69</v>
@@ -4214,7 +4533,6 @@
         <v>92</v>
       </c>
       <c r="AN11" s="29">
-        <f ca="1"/>
         <v>65017546092</v>
       </c>
       <c r="AO11" s="14" t="s">
@@ -4226,9 +4544,9 @@
       <c r="AQ11" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR11" s="19" t="str">
+      <c r="AR11" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS11" t="s">
         <v>96</v>
@@ -4258,10 +4576,10 @@
         <v>69</v>
       </c>
       <c r="BB11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="BC11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="BD11" s="14" t="s">
         <v>102</v>
@@ -4303,9 +4621,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13" t="s">
@@ -4318,10 +4636,10 @@
         <v>70</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I12" s="18">
         <v>25041111</v>
@@ -4333,7 +4651,7 @@
         <v>74</v>
       </c>
       <c r="L12" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M12" s="14" t="s">
@@ -4367,7 +4685,7 @@
         <v>74</v>
       </c>
       <c r="W12" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X12" s="18" t="s">
@@ -4380,7 +4698,7 @@
         <v>82</v>
       </c>
       <c r="AA12" s="25" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AB12" s="37" t="s">
         <v>135</v>
@@ -4410,7 +4728,7 @@
         <v>90</v>
       </c>
       <c r="AK12" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AL12" s="28" t="s">
         <v>69</v>
@@ -4419,7 +4737,6 @@
         <v>92</v>
       </c>
       <c r="AN12" s="29">
-        <f ca="1"/>
         <v>69463381017</v>
       </c>
       <c r="AO12" s="14" t="s">
@@ -4431,9 +4748,9 @@
       <c r="AQ12" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR12" s="19" t="str">
+      <c r="AR12" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS12" t="s">
         <v>96</v>
@@ -4505,12 +4822,12 @@
         <v>113</v>
       </c>
       <c r="BP12" s="38" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
-    <row r="13" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="13" t="s">
@@ -4523,10 +4840,10 @@
         <v>70</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I13" s="18">
         <v>25041111</v>
@@ -4538,7 +4855,7 @@
         <v>74</v>
       </c>
       <c r="L13" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M13" s="14" t="s">
@@ -4572,7 +4889,7 @@
         <v>74</v>
       </c>
       <c r="W13" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X13" s="18" t="s">
@@ -4585,7 +4902,7 @@
         <v>122</v>
       </c>
       <c r="AA13" s="25" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="AB13" s="37" t="s">
         <v>84</v>
@@ -4606,7 +4923,7 @@
         <v>87</v>
       </c>
       <c r="AH13" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46100</v>
       </c>
       <c r="AI13" s="18" t="s">
@@ -4616,7 +4933,7 @@
         <v>90</v>
       </c>
       <c r="AK13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AL13" s="28" t="s">
         <v>69</v>
@@ -4625,7 +4942,6 @@
         <v>92</v>
       </c>
       <c r="AN13" s="29">
-        <f ca="1"/>
         <v>68204494491</v>
       </c>
       <c r="AO13" s="14" t="s">
@@ -4638,7 +4954,7 @@
         <v>95</v>
       </c>
       <c r="AR13" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46100</v>
       </c>
       <c r="AS13" t="s">
@@ -4669,10 +4985,10 @@
         <v>69</v>
       </c>
       <c r="BB13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="BC13" s="34" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="BD13" s="14" t="s">
         <v>102</v>
@@ -4714,9 +5030,9 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="13" t="s">
@@ -4729,10 +5045,10 @@
         <v>70</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I14" s="18">
         <v>25041111</v>
@@ -4744,7 +5060,7 @@
         <v>74</v>
       </c>
       <c r="L14" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M14" s="14" t="s">
@@ -4778,7 +5094,7 @@
         <v>74</v>
       </c>
       <c r="W14" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X14" s="18" t="s">
@@ -4791,7 +5107,7 @@
         <v>82</v>
       </c>
       <c r="AA14" s="25" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AB14" s="37" t="s">
         <v>135</v>
@@ -4821,7 +5137,7 @@
         <v>90</v>
       </c>
       <c r="AK14" s="38" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AL14" s="28" t="s">
         <v>69</v>
@@ -4830,7 +5146,6 @@
         <v>92</v>
       </c>
       <c r="AN14" s="29">
-        <f ca="1"/>
         <v>24226361657</v>
       </c>
       <c r="AO14" s="14" t="s">
@@ -4842,9 +5157,9 @@
       <c r="AQ14" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR14" s="19" t="str">
+      <c r="AR14" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS14" t="s">
         <v>96</v>
@@ -4916,12 +5231,12 @@
         <v>113</v>
       </c>
       <c r="BP14" s="38" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
-    <row r="15" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="13" t="s">
@@ -4934,10 +5249,10 @@
         <v>70</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I15" s="18">
         <v>25041111</v>
@@ -4949,7 +5264,7 @@
         <v>74</v>
       </c>
       <c r="L15" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M15" s="14" t="s">
@@ -4983,7 +5298,7 @@
         <v>74</v>
       </c>
       <c r="W15" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X15" s="18" t="s">
@@ -5017,7 +5332,7 @@
         <v>87</v>
       </c>
       <c r="AH15" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46100</v>
       </c>
       <c r="AI15" s="18" t="s">
@@ -5036,7 +5351,6 @@
         <v>92</v>
       </c>
       <c r="AN15" s="29">
-        <f ca="1"/>
         <v>75635122197</v>
       </c>
       <c r="AO15" s="14" t="s">
@@ -5049,7 +5363,7 @@
         <v>95</v>
       </c>
       <c r="AR15" s="19">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>46100</v>
       </c>
       <c r="AS15" t="s">
@@ -5080,10 +5394,10 @@
         <v>69</v>
       </c>
       <c r="BB15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="BC15" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="BD15" s="14" t="s">
         <v>102</v>
@@ -5125,9 +5439,9 @@
         <v>153</v>
       </c>
     </row>
-    <row r="16" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
@@ -5140,10 +5454,10 @@
         <v>70</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I16" s="18">
         <v>25041111</v>
@@ -5155,7 +5469,7 @@
         <v>74</v>
       </c>
       <c r="L16" s="19">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45704</v>
       </c>
       <c r="M16" s="14" t="s">
@@ -5189,20 +5503,20 @@
         <v>74</v>
       </c>
       <c r="W16" s="23">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45704</v>
       </c>
       <c r="X16" s="18" t="s">
         <v>80</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Z16" s="38" t="s">
         <v>82</v>
       </c>
       <c r="AA16" s="25" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AB16" s="37" t="s">
         <v>84</v>
@@ -5241,7 +5555,6 @@
         <v>92</v>
       </c>
       <c r="AN16" s="29">
-        <f ca="1"/>
         <v>21045840423</v>
       </c>
       <c r="AO16" s="14" t="s">
@@ -5253,9 +5566,9 @@
       <c r="AQ16" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="AR16" s="19" t="str">
+      <c r="AR16" s="19">
         <f t="shared" si="4"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS16" t="s">
         <v>96</v>
@@ -5331,33 +5644,69 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ10:AQ16 X10:X16 V10:V16 S10:S16 K10:K16 BI10:BI16 AX10:AX16" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="14">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ10:AQ16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ16 X2:X16 V2:V16 S2:S16 K2:K16 BI2:BI16 AX2:AX16" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX10:AX16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI10:BI16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K10:K16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S10:S16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X10:X16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="U4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="U5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="U6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="U7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="U8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="U9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="U10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="U11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="U12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="U13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="U14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="U15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="U16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="U2" r:id="rId1"/>
+    <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U4" r:id="rId3"/>
+    <hyperlink ref="U5" r:id="rId4"/>
+    <hyperlink ref="U6" r:id="rId5"/>
+    <hyperlink ref="U7" r:id="rId6"/>
+    <hyperlink ref="U8" r:id="rId7"/>
+    <hyperlink ref="U9" r:id="rId8"/>
+    <hyperlink ref="U10" r:id="rId9"/>
+    <hyperlink ref="U11" r:id="rId10"/>
+    <hyperlink ref="U12" r:id="rId11"/>
+    <hyperlink ref="U13" r:id="rId12"/>
+    <hyperlink ref="U14" r:id="rId13"/>
+    <hyperlink ref="U15" r:id="rId14"/>
+    <hyperlink ref="U16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>